<commit_message>
feat: update review workflows and electron integration
</commit_message>
<xml_diff>
--- a/Thesis_progress_25_11_25.xlsx
+++ b/Thesis_progress_25_11_25.xlsx
@@ -16,7 +16,7 @@
     <definedName name="task_start" localSheetId="0">'Project schedule'!$D$9:$D$23</definedName>
     <definedName name="today" localSheetId="0">TODAY()</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Project schedule'!$4:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Project schedule'!$B$4:$BD$23</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Project schedule'!$H$4:$BF$23</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -31,7 +31,7 @@
     <numFmt numFmtId="167" formatCode="0_ ;[Red]\-0\ "/>
     <numFmt numFmtId="168" formatCode="ddd\,\ m/d/yyyy"/>
   </numFmts>
-  <fonts count="37">
+  <fonts count="73">
     <font>
       <name val="Arial"/>
       <family val="2"/>
@@ -283,6 +283,235 @@
       <b val="1"/>
       <color rgb="FF1F2937"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF1F2937"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Liberation Sans"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="7.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <color theme="0"/>
+      <sz val="22"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="24"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <sz val="22"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="22"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <color rgb="FF000000"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FF1F2937"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="20"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <sz val="20"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Liberation Sans"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF000000"/>
+      <sz val="18"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF1F2937"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF3F2A56"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF1F2937"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF7A1F5C"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <i val="1"/>
+      <color theme="1"/>
+      <sz val="20"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="18"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <color rgb="FF000000"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FF1F2937"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <sz val="14"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Liberation Sans"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF1F2937"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <i val="1"/>
+      <color theme="1"/>
+      <sz val="14"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <i val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FF1F2937"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Liberation Sans"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF000000"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF1F2937"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF3F2A56"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF7A1F5C"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="12">
@@ -348,7 +577,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="50">
+  <borders count="53">
     <border>
       <left/>
       <right/>
@@ -927,6 +1156,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color theme="1"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color theme="1"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color theme="1"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="11">
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
@@ -954,7 +1210,7 @@
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="145">
+  <cellXfs count="294">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1309,6 +1565,383 @@
     </xf>
     <xf numFmtId="0" fontId="36" fillId="0" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="34" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="5">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="34" fillId="6" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="35" fillId="2" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="34" fillId="0" borderId="51" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="5">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="52" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="36" fillId="0" borderId="51" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="5">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="26" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="40" fillId="7" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="42" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="50" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="43" fillId="8" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="43" fillId="8" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="42" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="8">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="3"/>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="9" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="40" fillId="9" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="40" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="45" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="10">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="9" fontId="46" fillId="10" borderId="37" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="10" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="40" fillId="10" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="42" fillId="0" borderId="39" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="8">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="39" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="46" fillId="3" borderId="37" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="54" fillId="7" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="54" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="14" fontId="55" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="50" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="56" fillId="8" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="56" fillId="8" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="8">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="9" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="54" fillId="9" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="54" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="10">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="9" fontId="58" fillId="10" borderId="37" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="60" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="60" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="10" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="54" fillId="10" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="39" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="8">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="61" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="58" fillId="3" borderId="37" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="50" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="62" fillId="8" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="62" fillId="8" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="64" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="65" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="65" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="65" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="64" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="65" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="65" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="65" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="65" fillId="0" borderId="50" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="65" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="10">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="10" borderId="37" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="66" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="65" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="67" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="68" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="69" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="68" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="70" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="65" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="63" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="3" borderId="37" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="65" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="71" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="71" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="71" fillId="0" borderId="50" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="71" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="71" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="71" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="68" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="71" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="71" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="71" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="72" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="71" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="71" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="11">
@@ -1324,7 +1957,7 @@
     <cellStyle name="Name" xfId="9"/>
     <cellStyle name="Task" xfId="10"/>
   </cellStyles>
-  <dxfs count="13">
+  <dxfs count="15">
     <dxf>
       <border>
         <left style="thin">
@@ -1441,6 +2074,20 @@
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="FFFFD6F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFF66CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC2E8"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1828,69 +2475,69 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName="Sheet1">
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BP27"/>
+  <dimension ref="A1:CA27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.75" defaultRowHeight="30" customHeight="1"/>
   <cols>
     <col width="2.75" customWidth="1" style="130" min="1" max="1"/>
-    <col width="22.75" customWidth="1" style="127" min="2" max="2"/>
-    <col width="10.75" customWidth="1" style="127" min="3" max="3"/>
-    <col width="10.75" customWidth="1" style="44" min="4" max="4"/>
-    <col width="10.75" customWidth="1" style="49" min="5" max="5"/>
-    <col width="2.75" customWidth="1" style="127" min="6" max="6"/>
-    <col width="6" customWidth="1" style="127" min="7" max="7"/>
-    <col width="2" customWidth="1" style="127" min="8" max="56"/>
-    <col width="2.5" customWidth="1" style="127" min="9" max="9"/>
-    <col width="2.5" customWidth="1" style="127" min="10" max="10"/>
-    <col width="2.5" customWidth="1" style="127" min="11" max="11"/>
-    <col width="2.5" customWidth="1" style="127" min="12" max="12"/>
-    <col width="2.5" customWidth="1" style="127" min="13" max="13"/>
-    <col width="2.5" customWidth="1" style="127" min="14" max="14"/>
-    <col width="2.5" customWidth="1" style="127" min="15" max="15"/>
-    <col width="2.5" customWidth="1" style="127" min="16" max="16"/>
-    <col width="2.5" customWidth="1" style="127" min="17" max="17"/>
-    <col width="2.5" customWidth="1" style="127" min="18" max="18"/>
-    <col width="2.5" customWidth="1" style="127" min="19" max="19"/>
-    <col width="2.5" customWidth="1" style="127" min="20" max="20"/>
-    <col width="2.5" customWidth="1" style="127" min="21" max="21"/>
-    <col width="2.5" customWidth="1" style="127" min="22" max="22"/>
-    <col width="2.5" customWidth="1" style="127" min="23" max="23"/>
-    <col width="2.5" customWidth="1" style="127" min="24" max="24"/>
-    <col width="2.5" customWidth="1" style="127" min="25" max="25"/>
-    <col width="2.5" customWidth="1" style="127" min="26" max="26"/>
-    <col width="2.5" customWidth="1" style="127" min="27" max="27"/>
-    <col width="2.5" customWidth="1" style="127" min="28" max="28"/>
-    <col width="2.5" customWidth="1" style="127" min="29" max="29"/>
-    <col width="2.5" customWidth="1" style="127" min="30" max="30"/>
-    <col width="2.5" customWidth="1" style="127" min="31" max="31"/>
-    <col width="2.5" customWidth="1" style="127" min="32" max="32"/>
-    <col width="2.5" customWidth="1" style="127" min="33" max="33"/>
-    <col width="2.5" customWidth="1" style="127" min="34" max="34"/>
-    <col width="2.5" customWidth="1" style="127" min="35" max="35"/>
-    <col width="2.5" customWidth="1" style="127" min="36" max="36"/>
-    <col width="2.5" customWidth="1" style="127" min="37" max="37"/>
-    <col width="2.5" customWidth="1" style="127" min="38" max="38"/>
-    <col width="2.5" customWidth="1" style="127" min="39" max="39"/>
-    <col width="2.5" customWidth="1" style="127" min="40" max="40"/>
-    <col width="2.5" customWidth="1" style="127" min="41" max="41"/>
-    <col width="2.5" customWidth="1" style="127" min="42" max="42"/>
-    <col width="2.5" customWidth="1" style="127" min="43" max="43"/>
-    <col width="2.5" customWidth="1" style="127" min="44" max="44"/>
-    <col width="2.5" customWidth="1" style="127" min="45" max="45"/>
-    <col width="2.5" customWidth="1" style="127" min="46" max="46"/>
-    <col width="2.5" customWidth="1" style="127" min="47" max="47"/>
-    <col width="2.5" customWidth="1" style="127" min="48" max="48"/>
-    <col width="2.5" customWidth="1" style="127" min="49" max="49"/>
-    <col width="2.5" customWidth="1" style="127" min="50" max="50"/>
-    <col width="2.5" customWidth="1" style="127" min="51" max="51"/>
-    <col width="2.5" customWidth="1" style="127" min="52" max="52"/>
-    <col width="2.5" customWidth="1" style="127" min="53" max="53"/>
-    <col width="2.5" customWidth="1" style="127" min="54" max="54"/>
-    <col width="2.5" customWidth="1" style="127" min="55" max="55"/>
-    <col width="2.5" customWidth="1" style="127" min="56" max="56"/>
-    <col hidden="1" width="2.75" customWidth="1" style="127" min="57" max="57"/>
-    <col hidden="1" width="13" customWidth="1" style="127" min="58" max="64"/>
+    <col width="36" customWidth="1" style="127" min="2" max="2"/>
+    <col hidden="1" width="10.75" customWidth="1" style="127" min="3" max="3"/>
+    <col hidden="1" width="10.75" customWidth="1" style="44" min="4" max="4"/>
+    <col hidden="1" width="10.75" customWidth="1" style="49" min="5" max="5"/>
+    <col hidden="1" width="2.75" customWidth="1" style="127" min="6" max="6"/>
+    <col hidden="1" width="6" customWidth="1" style="127" min="7" max="7"/>
+    <col width="2.38" customWidth="1" style="127" min="8" max="56"/>
+    <col width="2.38" customWidth="1" style="127" min="9" max="9"/>
+    <col width="2.38" customWidth="1" style="127" min="10" max="10"/>
+    <col width="2.38" customWidth="1" style="127" min="11" max="11"/>
+    <col width="2.38" customWidth="1" style="127" min="12" max="12"/>
+    <col width="2.38" customWidth="1" style="127" min="13" max="13"/>
+    <col width="2.38" customWidth="1" style="127" min="14" max="14"/>
+    <col width="2.38" customWidth="1" style="127" min="15" max="15"/>
+    <col width="2.38" customWidth="1" style="127" min="16" max="16"/>
+    <col width="2.38" customWidth="1" style="127" min="17" max="17"/>
+    <col width="2.38" customWidth="1" style="127" min="18" max="18"/>
+    <col width="2.38" customWidth="1" style="127" min="19" max="19"/>
+    <col width="2.38" customWidth="1" style="127" min="20" max="20"/>
+    <col width="2.38" customWidth="1" style="127" min="21" max="21"/>
+    <col width="2.38" customWidth="1" style="127" min="22" max="22"/>
+    <col width="2.38" customWidth="1" style="127" min="23" max="23"/>
+    <col width="2.38" customWidth="1" style="127" min="24" max="24"/>
+    <col width="2.38" customWidth="1" style="127" min="25" max="25"/>
+    <col width="2.38" customWidth="1" style="127" min="26" max="26"/>
+    <col width="2.38" customWidth="1" style="127" min="27" max="27"/>
+    <col width="2.38" customWidth="1" style="127" min="28" max="28"/>
+    <col width="2.38" customWidth="1" style="127" min="29" max="29"/>
+    <col width="2.38" customWidth="1" style="127" min="30" max="30"/>
+    <col width="2.38" customWidth="1" style="127" min="31" max="31"/>
+    <col width="2.38" customWidth="1" style="127" min="32" max="32"/>
+    <col width="2.38" customWidth="1" style="127" min="33" max="33"/>
+    <col width="2.38" customWidth="1" style="127" min="34" max="34"/>
+    <col width="2.38" customWidth="1" style="127" min="35" max="35"/>
+    <col width="2.38" customWidth="1" style="127" min="36" max="36"/>
+    <col width="2.38" customWidth="1" style="127" min="37" max="37"/>
+    <col width="2.38" customWidth="1" style="127" min="38" max="38"/>
+    <col width="2.38" customWidth="1" style="127" min="39" max="39"/>
+    <col width="2.38" customWidth="1" style="127" min="40" max="40"/>
+    <col width="2.38" customWidth="1" style="127" min="41" max="41"/>
+    <col width="2.38" customWidth="1" style="127" min="42" max="42"/>
+    <col width="2.38" customWidth="1" style="127" min="43" max="43"/>
+    <col width="2.38" customWidth="1" style="127" min="44" max="44"/>
+    <col width="2.38" customWidth="1" style="127" min="45" max="45"/>
+    <col width="2.38" customWidth="1" style="127" min="46" max="46"/>
+    <col width="2.38" customWidth="1" style="127" min="47" max="47"/>
+    <col width="2.38" customWidth="1" style="127" min="48" max="48"/>
+    <col width="2.38" customWidth="1" style="127" min="49" max="49"/>
+    <col width="2.38" customWidth="1" style="127" min="50" max="50"/>
+    <col width="2.38" customWidth="1" style="127" min="51" max="51"/>
+    <col width="2.38" customWidth="1" style="127" min="52" max="52"/>
+    <col width="2.38" customWidth="1" style="127" min="53" max="53"/>
+    <col width="2.38" customWidth="1" style="127" min="54" max="54"/>
+    <col width="2.38" customWidth="1" style="127" min="55" max="55"/>
+    <col width="2.38" customWidth="1" style="127" min="56" max="56"/>
+    <col width="2.38" customWidth="1" style="127" min="57" max="57"/>
+    <col width="2.38" customWidth="1" style="127" min="58" max="64"/>
     <col hidden="1" width="13" customWidth="1" style="127" min="59" max="59"/>
     <col hidden="1" width="13" customWidth="1" style="127" min="60" max="60"/>
     <col hidden="1" width="13" customWidth="1" style="127" min="61" max="61"/>
@@ -2119,81 +2766,44 @@
         </is>
       </c>
       <c r="G4" s="72" t="n"/>
-      <c r="H4" s="123">
+      <c r="H4" s="152">
         <f>IF(MONTH(H6)=9, YEAR(H6), "")</f>
         <v/>
       </c>
-      <c r="I4" s="124" t="n"/>
-      <c r="J4" s="124" t="n"/>
-      <c r="K4" s="125" t="n"/>
-      <c r="L4" s="123">
+      <c r="L4" s="152">
         <f>IF(MONTH(T6)=9, YEAR(T6), "")</f>
         <v/>
       </c>
-      <c r="M4" s="124" t="n"/>
-      <c r="N4" s="124" t="n"/>
-      <c r="O4" s="124" t="n"/>
-      <c r="P4" s="124" t="n"/>
-      <c r="Q4" s="124" t="n"/>
-      <c r="R4" s="124" t="n"/>
-      <c r="S4" s="124" t="n"/>
-      <c r="T4" s="124" t="n"/>
-      <c r="U4" s="124" t="n"/>
-      <c r="V4" s="124" t="n"/>
-      <c r="W4" s="125" t="n"/>
-      <c r="X4" s="123">
+      <c r="X4" s="152">
         <f>IF(MONTH(AF6)=9, YEAR(AF6), "")</f>
         <v/>
       </c>
-      <c r="Y4" s="124" t="n"/>
-      <c r="Z4" s="124" t="n"/>
-      <c r="AA4" s="124" t="n"/>
-      <c r="AB4" s="124" t="n"/>
-      <c r="AC4" s="124" t="n"/>
-      <c r="AD4" s="124" t="n"/>
-      <c r="AE4" s="124" t="n"/>
-      <c r="AF4" s="124" t="n"/>
-      <c r="AG4" s="124" t="n"/>
-      <c r="AH4" s="124" t="n"/>
-      <c r="AI4" s="125" t="n"/>
-      <c r="AJ4" s="123">
+      <c r="AJ4" s="152">
         <f>IF(MONTH(AR6)=9, YEAR(AR6), "")</f>
         <v/>
       </c>
-      <c r="AK4" s="124" t="n"/>
-      <c r="AL4" s="124" t="n"/>
-      <c r="AM4" s="124" t="n"/>
-      <c r="AN4" s="124" t="n"/>
-      <c r="AO4" s="124" t="n"/>
-      <c r="AP4" s="124" t="n"/>
-      <c r="AQ4" s="124" t="n"/>
-      <c r="AR4" s="124" t="n"/>
-      <c r="AS4" s="124" t="n"/>
-      <c r="AT4" s="124" t="n"/>
-      <c r="AU4" s="125" t="n"/>
-      <c r="AV4" s="123">
-        <f>IF(MONTH(BD6)=9, YEAR(BD6), "")</f>
-        <v/>
-      </c>
-      <c r="AW4" s="124" t="n"/>
-      <c r="AX4" s="124" t="n"/>
-      <c r="AY4" s="124" t="n"/>
-      <c r="AZ4" s="124" t="n"/>
-      <c r="BA4" s="124" t="n"/>
-      <c r="BB4" s="124" t="n"/>
-      <c r="BC4" s="124" t="n"/>
-      <c r="BD4" s="124" t="n"/>
-      <c r="BE4" s="124" t="n"/>
-      <c r="BF4" s="124" t="n"/>
-      <c r="BG4" s="125" t="n"/>
-      <c r="BH4" s="61" t="n"/>
-      <c r="BI4" s="52" t="n"/>
-      <c r="BJ4" s="52" t="n"/>
-      <c r="BK4" s="52" t="n"/>
-      <c r="BL4" s="52" t="n"/>
-      <c r="BM4" s="52" t="n"/>
-      <c r="BN4" s="52" t="n"/>
-      <c r="BO4" s="52" t="n"/>
+      <c r="AV4" s="171" t="n"/>
+      <c r="BG4" s="153" t="n"/>
+      <c r="BH4" s="172" t="n"/>
+      <c r="BI4" s="172" t="n"/>
+      <c r="BJ4" s="172" t="n"/>
+      <c r="BK4" s="172" t="n"/>
+      <c r="BL4" s="172" t="n"/>
+      <c r="BM4" s="172" t="n"/>
+      <c r="BN4" s="172" t="n"/>
+      <c r="BO4" s="172" t="n"/>
+      <c r="BP4" s="153" t="n"/>
+      <c r="BQ4" s="153" t="n"/>
+      <c r="BR4" s="153" t="n"/>
+      <c r="BS4" s="153" t="n"/>
+      <c r="BT4" s="153" t="n"/>
+      <c r="BU4" s="153" t="n"/>
+      <c r="BV4" s="153" t="n"/>
+      <c r="BW4" s="153" t="n"/>
+      <c r="BX4" s="153" t="n"/>
+      <c r="BY4" s="153" t="n"/>
+      <c r="BZ4" s="153" t="n"/>
+      <c r="CA4" s="153" t="n"/>
     </row>
     <row r="5" ht="14" customHeight="1" s="127" thickBot="1">
       <c r="A5" s="129" t="n"/>
@@ -2223,213 +2833,234 @@
         </is>
       </c>
       <c r="G5" s="102" t="n"/>
-      <c r="H5" s="113">
+      <c r="H5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:H5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="I5" s="113">
+      <c r="I5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:I5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="J5" s="113">
+      <c r="J5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:J5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="K5" s="113">
+      <c r="K5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:K5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="L5" s="113">
+      <c r="L5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:L5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="M5" s="113">
+      <c r="M5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:M5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="N5" s="113">
+      <c r="N5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:N5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="O5" s="113">
+      <c r="O5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:O5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="P5" s="113">
+      <c r="P5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:P5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="Q5" s="113">
+      <c r="Q5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:Q5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="R5" s="113">
+      <c r="R5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:R5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="S5" s="113">
+      <c r="S5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:S5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="T5" s="113">
+      <c r="T5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:T5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="U5" s="113">
+      <c r="U5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:U5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="V5" s="113">
+      <c r="V5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:V5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="W5" s="113">
+      <c r="W5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:W5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="X5" s="113">
+      <c r="X5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:X5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="Y5" s="113">
+      <c r="Y5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:Y5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="Z5" s="113">
+      <c r="Z5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:Z5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="AA5" s="113">
+      <c r="AA5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:AA5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="AB5" s="113">
+      <c r="AB5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:AB5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="AC5" s="113">
+      <c r="AC5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:AC5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="AD5" s="113">
+      <c r="AD5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:AD5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="AE5" s="113">
+      <c r="AE5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:AE5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="AF5" s="113">
+      <c r="AF5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:AF5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="AG5" s="113">
+      <c r="AG5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:AG5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="AH5" s="113">
+      <c r="AH5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:AH5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="AI5" s="113">
+      <c r="AI5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:AI5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="AJ5" s="113">
+      <c r="AJ5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:AJ5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="AK5" s="113">
+      <c r="AK5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:AK5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="AL5" s="113">
+      <c r="AL5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:AL5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="AM5" s="113">
+      <c r="AM5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:AM5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="AN5" s="113">
+      <c r="AN5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:AN5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="AO5" s="113">
+      <c r="AO5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:AO5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="AP5" s="113">
+      <c r="AP5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:AP5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="AQ5" s="113">
+      <c r="AQ5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:AQ5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="AR5" s="113">
+      <c r="AR5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:AR5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="AS5" s="113">
+      <c r="AS5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:AS5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="AT5" s="113">
+      <c r="AT5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:AT5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="AU5" s="113">
+      <c r="AU5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:AU5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="AV5" s="113">
+      <c r="AV5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:AV5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="AW5" s="113">
+      <c r="AW5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:AW5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="AX5" s="113">
+      <c r="AX5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:AX5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="AY5" s="113">
+      <c r="AY5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:AY5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="AZ5" s="113">
+      <c r="AZ5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:AZ5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="BA5" s="113">
+      <c r="BA5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:BA5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="BB5" s="113">
+      <c r="BB5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:BB5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="BC5" s="113">
+      <c r="BC5" s="154">
         <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:BC5)-1), "mmm"), 1)</f>
         <v/>
       </c>
-      <c r="BD5" s="113">
-        <f>LEFT(TEXT(EDATE(Project_Start, COLUMNS($H5:BD5)-1), "mmm"), 1)</f>
-        <v/>
-      </c>
-      <c r="BE5" s="39" t="n"/>
-      <c r="BF5" s="39" t="n"/>
-      <c r="BG5" s="73" t="n"/>
-      <c r="BH5" s="87" t="n"/>
-      <c r="BI5" s="39" t="n"/>
-      <c r="BJ5" s="39" t="n"/>
-      <c r="BK5" s="39" t="n"/>
-      <c r="BL5" s="39" t="n"/>
-      <c r="BM5" s="39" t="n"/>
-      <c r="BN5" s="39" t="n"/>
-      <c r="BO5" s="39" t="n"/>
+      <c r="BD5" s="154" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BE5" s="154" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="BF5" s="154" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="BG5" s="173" t="n"/>
+      <c r="BH5" s="173" t="n"/>
+      <c r="BI5" s="173" t="n"/>
+      <c r="BJ5" s="173" t="n"/>
+      <c r="BK5" s="173" t="n"/>
+      <c r="BL5" s="173" t="n"/>
+      <c r="BM5" s="173" t="n"/>
+      <c r="BN5" s="173" t="n"/>
+      <c r="BO5" s="173" t="n"/>
+      <c r="BP5" s="153" t="n"/>
+      <c r="BQ5" s="153" t="n"/>
+      <c r="BR5" s="153" t="n"/>
+      <c r="BS5" s="153" t="n"/>
+      <c r="BT5" s="153" t="n"/>
+      <c r="BU5" s="153" t="n"/>
+      <c r="BV5" s="153" t="n"/>
+      <c r="BW5" s="153" t="n"/>
+      <c r="BX5" s="153" t="n"/>
+      <c r="BY5" s="153" t="n"/>
+      <c r="BZ5" s="153" t="n"/>
+      <c r="CA5" s="153" t="n"/>
     </row>
     <row r="6" hidden="1" ht="14" customHeight="1" s="127" thickBot="1">
       <c r="B6" s="122" t="n"/>
@@ -2442,213 +3073,231 @@
         </is>
       </c>
       <c r="G6" s="103" t="n"/>
-      <c r="H6" s="114">
+      <c r="H6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:H6)-1)</f>
         <v/>
       </c>
-      <c r="I6" s="114">
+      <c r="I6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:I6)-1)</f>
         <v/>
       </c>
-      <c r="J6" s="114">
+      <c r="J6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:J6)-1)</f>
         <v/>
       </c>
-      <c r="K6" s="114">
+      <c r="K6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:K6)-1)</f>
         <v/>
       </c>
-      <c r="L6" s="114">
+      <c r="L6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:L6)-1)</f>
         <v/>
       </c>
-      <c r="M6" s="114">
+      <c r="M6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:M6)-1)</f>
         <v/>
       </c>
-      <c r="N6" s="114">
+      <c r="N6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:N6)-1)</f>
         <v/>
       </c>
-      <c r="O6" s="114">
+      <c r="O6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:O6)-1)</f>
         <v/>
       </c>
-      <c r="P6" s="114">
+      <c r="P6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:P6)-1)</f>
         <v/>
       </c>
-      <c r="Q6" s="114">
+      <c r="Q6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:Q6)-1)</f>
         <v/>
       </c>
-      <c r="R6" s="114">
+      <c r="R6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:R6)-1)</f>
         <v/>
       </c>
-      <c r="S6" s="114">
+      <c r="S6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:S6)-1)</f>
         <v/>
       </c>
-      <c r="T6" s="114">
+      <c r="T6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:T6)-1)</f>
         <v/>
       </c>
-      <c r="U6" s="114">
+      <c r="U6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:U6)-1)</f>
         <v/>
       </c>
-      <c r="V6" s="114">
+      <c r="V6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:V6)-1)</f>
         <v/>
       </c>
-      <c r="W6" s="114">
+      <c r="W6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:W6)-1)</f>
         <v/>
       </c>
-      <c r="X6" s="114">
+      <c r="X6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:X6)-1)</f>
         <v/>
       </c>
-      <c r="Y6" s="114">
+      <c r="Y6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:Y6)-1)</f>
         <v/>
       </c>
-      <c r="Z6" s="114">
+      <c r="Z6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:Z6)-1)</f>
         <v/>
       </c>
-      <c r="AA6" s="114">
+      <c r="AA6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:AA6)-1)</f>
         <v/>
       </c>
-      <c r="AB6" s="114">
+      <c r="AB6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:AB6)-1)</f>
         <v/>
       </c>
-      <c r="AC6" s="114">
+      <c r="AC6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:AC6)-1)</f>
         <v/>
       </c>
-      <c r="AD6" s="114">
+      <c r="AD6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:AD6)-1)</f>
         <v/>
       </c>
-      <c r="AE6" s="114">
+      <c r="AE6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:AE6)-1)</f>
         <v/>
       </c>
-      <c r="AF6" s="114">
+      <c r="AF6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:AF6)-1)</f>
         <v/>
       </c>
-      <c r="AG6" s="114">
+      <c r="AG6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:AG6)-1)</f>
         <v/>
       </c>
-      <c r="AH6" s="114">
+      <c r="AH6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:AH6)-1)</f>
         <v/>
       </c>
-      <c r="AI6" s="114">
+      <c r="AI6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:AI6)-1)</f>
         <v/>
       </c>
-      <c r="AJ6" s="114">
+      <c r="AJ6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:AJ6)-1)</f>
         <v/>
       </c>
-      <c r="AK6" s="114">
+      <c r="AK6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:AK6)-1)</f>
         <v/>
       </c>
-      <c r="AL6" s="114">
+      <c r="AL6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:AL6)-1)</f>
         <v/>
       </c>
-      <c r="AM6" s="114">
+      <c r="AM6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:AM6)-1)</f>
         <v/>
       </c>
-      <c r="AN6" s="114">
+      <c r="AN6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:AN6)-1)</f>
         <v/>
       </c>
-      <c r="AO6" s="114">
+      <c r="AO6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:AO6)-1)</f>
         <v/>
       </c>
-      <c r="AP6" s="114">
+      <c r="AP6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:AP6)-1)</f>
         <v/>
       </c>
-      <c r="AQ6" s="114">
+      <c r="AQ6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:AQ6)-1)</f>
         <v/>
       </c>
-      <c r="AR6" s="114">
+      <c r="AR6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:AR6)-1)</f>
         <v/>
       </c>
-      <c r="AS6" s="114">
+      <c r="AS6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:AS6)-1)</f>
         <v/>
       </c>
-      <c r="AT6" s="114">
+      <c r="AT6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:AT6)-1)</f>
         <v/>
       </c>
-      <c r="AU6" s="114">
+      <c r="AU6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:AU6)-1)</f>
         <v/>
       </c>
-      <c r="AV6" s="114">
+      <c r="AV6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:AV6)-1)</f>
         <v/>
       </c>
-      <c r="AW6" s="114">
+      <c r="AW6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:AW6)-1)</f>
         <v/>
       </c>
-      <c r="AX6" s="114">
+      <c r="AX6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:AX6)-1)</f>
         <v/>
       </c>
-      <c r="AY6" s="114">
+      <c r="AY6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:AY6)-1)</f>
         <v/>
       </c>
-      <c r="AZ6" s="114">
+      <c r="AZ6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:AZ6)-1)</f>
         <v/>
       </c>
-      <c r="BA6" s="114">
+      <c r="BA6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:BA6)-1)</f>
         <v/>
       </c>
-      <c r="BB6" s="114">
+      <c r="BB6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:BB6)-1)</f>
         <v/>
       </c>
-      <c r="BC6" s="114">
+      <c r="BC6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:BC6)-1)</f>
         <v/>
       </c>
-      <c r="BD6" s="114">
+      <c r="BD6" s="155">
         <f>EDATE(Project_Start, COLUMNS($H6:BD6)-1)</f>
         <v/>
       </c>
-      <c r="BE6" s="51" t="n"/>
-      <c r="BF6" s="51" t="n"/>
-      <c r="BG6" s="74" t="n"/>
-      <c r="BH6" s="51" t="n"/>
-      <c r="BI6" s="51" t="n"/>
-      <c r="BJ6" s="51" t="n"/>
-      <c r="BK6" s="51" t="n"/>
-      <c r="BL6" s="51" t="n"/>
-      <c r="BM6" s="51" t="n"/>
-      <c r="BN6" s="51" t="n"/>
-      <c r="BO6" s="51" t="n"/>
+      <c r="BE6" s="155">
+        <f>EDATE(Project_Start, COLUMNS($H6:BE6)-1)</f>
+        <v/>
+      </c>
+      <c r="BF6" s="155">
+        <f>EDATE(Project_Start, COLUMNS($H6:BF6)-1)</f>
+        <v/>
+      </c>
+      <c r="BG6" s="174" t="n"/>
+      <c r="BH6" s="174" t="n"/>
+      <c r="BI6" s="174" t="n"/>
+      <c r="BJ6" s="174" t="n"/>
+      <c r="BK6" s="174" t="n"/>
+      <c r="BL6" s="174" t="n"/>
+      <c r="BM6" s="174" t="n"/>
+      <c r="BN6" s="174" t="n"/>
+      <c r="BO6" s="174" t="n"/>
+      <c r="BP6" s="153" t="n"/>
+      <c r="BQ6" s="153" t="n"/>
+      <c r="BR6" s="153" t="n"/>
+      <c r="BS6" s="153" t="n"/>
+      <c r="BT6" s="153" t="n"/>
+      <c r="BU6" s="153" t="n"/>
+      <c r="BV6" s="153" t="n"/>
+      <c r="BW6" s="153" t="n"/>
+      <c r="BX6" s="153" t="n"/>
+      <c r="BY6" s="153" t="n"/>
+      <c r="BZ6" s="153" t="n"/>
+      <c r="CA6" s="153" t="n"/>
     </row>
     <row r="7" hidden="1" ht="20" customHeight="1" s="127">
       <c r="A7" s="130" t="inlineStr">
@@ -2664,127 +3313,179 @@
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v/>
       </c>
-      <c r="H7" s="58" t="n"/>
-      <c r="I7" s="58" t="n"/>
-      <c r="J7" s="58" t="n"/>
-      <c r="K7" s="58" t="n"/>
-      <c r="L7" s="58" t="n"/>
-      <c r="M7" s="58" t="n"/>
-      <c r="N7" s="58" t="n"/>
-      <c r="O7" s="58" t="n"/>
-      <c r="P7" s="58" t="n"/>
-      <c r="Q7" s="58" t="n"/>
-      <c r="R7" s="58" t="n"/>
-      <c r="S7" s="58" t="n"/>
-      <c r="T7" s="58" t="n"/>
-      <c r="U7" s="58" t="n"/>
-      <c r="V7" s="58" t="n"/>
-      <c r="W7" s="58" t="n"/>
-      <c r="X7" s="58" t="n"/>
-      <c r="Y7" s="58" t="n"/>
-      <c r="Z7" s="58" t="n"/>
-      <c r="AA7" s="58" t="n"/>
-      <c r="AB7" s="58" t="n"/>
-      <c r="AC7" s="58" t="n"/>
-      <c r="AD7" s="58" t="n"/>
-      <c r="AE7" s="58" t="n"/>
-      <c r="AF7" s="58" t="n"/>
-      <c r="AG7" s="58" t="n"/>
-      <c r="AH7" s="58" t="n"/>
-      <c r="AI7" s="58" t="n"/>
-      <c r="AJ7" s="58" t="n"/>
-      <c r="AK7" s="58" t="n"/>
-      <c r="AL7" s="58" t="n"/>
-      <c r="AM7" s="58" t="n"/>
-      <c r="AN7" s="58" t="n"/>
-      <c r="AO7" s="58" t="n"/>
-      <c r="AP7" s="57" t="n"/>
-      <c r="AQ7" s="53" t="n"/>
-      <c r="AR7" s="53" t="n"/>
-      <c r="AS7" s="53" t="n"/>
-      <c r="AT7" s="53" t="n"/>
-      <c r="AU7" s="53" t="n"/>
-      <c r="AV7" s="53" t="n"/>
-      <c r="AW7" s="53" t="n"/>
-      <c r="AX7" s="53" t="n"/>
-      <c r="AY7" s="53" t="n"/>
-      <c r="AZ7" s="53" t="n"/>
-      <c r="BA7" s="53" t="n"/>
-      <c r="BB7" s="53" t="n"/>
-      <c r="BC7" s="53" t="n"/>
-      <c r="BD7" s="53" t="n"/>
+      <c r="H7" s="156" t="n"/>
+      <c r="I7" s="156" t="n"/>
+      <c r="J7" s="156" t="n"/>
+      <c r="K7" s="156" t="n"/>
+      <c r="L7" s="156" t="n"/>
+      <c r="M7" s="156" t="n"/>
+      <c r="N7" s="156" t="n"/>
+      <c r="O7" s="156" t="n"/>
+      <c r="P7" s="156" t="n"/>
+      <c r="Q7" s="156" t="n"/>
+      <c r="R7" s="156" t="n"/>
+      <c r="S7" s="156" t="n"/>
+      <c r="T7" s="156" t="n"/>
+      <c r="U7" s="156" t="n"/>
+      <c r="V7" s="156" t="n"/>
+      <c r="W7" s="156" t="n"/>
+      <c r="X7" s="156" t="n"/>
+      <c r="Y7" s="156" t="n"/>
+      <c r="Z7" s="156" t="n"/>
+      <c r="AA7" s="156" t="n"/>
+      <c r="AB7" s="156" t="n"/>
+      <c r="AC7" s="156" t="n"/>
+      <c r="AD7" s="156" t="n"/>
+      <c r="AE7" s="156" t="n"/>
+      <c r="AF7" s="156" t="n"/>
+      <c r="AG7" s="156" t="n"/>
+      <c r="AH7" s="156" t="n"/>
+      <c r="AI7" s="156" t="n"/>
+      <c r="AJ7" s="156" t="n"/>
+      <c r="AK7" s="156" t="n"/>
+      <c r="AL7" s="156" t="n"/>
+      <c r="AM7" s="156" t="n"/>
+      <c r="AN7" s="156" t="n"/>
+      <c r="AO7" s="156" t="n"/>
+      <c r="AP7" s="156" t="n"/>
+      <c r="AQ7" s="156" t="n"/>
+      <c r="AR7" s="156" t="n"/>
+      <c r="AS7" s="156" t="n"/>
+      <c r="AT7" s="156" t="n"/>
+      <c r="AU7" s="156" t="n"/>
+      <c r="AV7" s="156" t="n"/>
+      <c r="AW7" s="156" t="n"/>
+      <c r="AX7" s="156" t="n"/>
+      <c r="AY7" s="156" t="n"/>
+      <c r="AZ7" s="156" t="n"/>
+      <c r="BA7" s="156" t="n"/>
+      <c r="BB7" s="156" t="n"/>
+      <c r="BC7" s="156" t="n"/>
+      <c r="BD7" s="156" t="n"/>
       <c r="BE7" s="53" t="n"/>
       <c r="BF7" s="53" t="n"/>
-      <c r="BG7" s="77" t="n"/>
-      <c r="BH7" s="53" t="n"/>
-      <c r="BI7" s="53" t="n"/>
-      <c r="BJ7" s="53" t="n"/>
-      <c r="BK7" s="53" t="n"/>
+      <c r="BG7" s="156" t="n"/>
+      <c r="BH7" s="156" t="n"/>
+      <c r="BI7" s="156" t="n"/>
+      <c r="BJ7" s="156" t="n"/>
+      <c r="BK7" s="156" t="n"/>
+      <c r="BL7" s="153" t="n"/>
+      <c r="BM7" s="153" t="n"/>
+      <c r="BN7" s="153" t="n"/>
+      <c r="BO7" s="153" t="n"/>
+      <c r="BP7" s="153" t="n"/>
+      <c r="BQ7" s="153" t="n"/>
+      <c r="BR7" s="153" t="n"/>
+      <c r="BS7" s="153" t="n"/>
+      <c r="BT7" s="153" t="n"/>
+      <c r="BU7" s="153" t="n"/>
+      <c r="BV7" s="153" t="n"/>
+      <c r="BW7" s="153" t="n"/>
+      <c r="BX7" s="153" t="n"/>
+      <c r="BY7" s="153" t="n"/>
+      <c r="BZ7" s="153" t="n"/>
+      <c r="CA7" s="153" t="n"/>
     </row>
-    <row r="8" ht="20" customFormat="1" customHeight="1" s="53" thickBot="1">
-      <c r="A8" s="129" t="n"/>
-      <c r="B8" s="91" t="inlineStr">
+    <row r="8" ht="46" customFormat="1" customHeight="1" s="53" thickBot="1">
+      <c r="A8" s="178" t="n"/>
+      <c r="B8" s="221" t="inlineStr">
         <is>
           <t>Phase 1 - Preliminary Research</t>
         </is>
       </c>
-      <c r="C8" s="92" t="inlineStr">
+      <c r="C8" s="222" t="inlineStr">
         <is>
           <t>Phase 1: Preliminary Research</t>
         </is>
       </c>
-      <c r="D8" s="89" t="n"/>
-      <c r="E8" s="89" t="n"/>
-      <c r="F8" s="13" t="n"/>
-      <c r="G8" s="3">
+      <c r="D8" s="223" t="n"/>
+      <c r="E8" s="223" t="n"/>
+      <c r="F8" s="182" t="n"/>
+      <c r="G8" s="183">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v/>
       </c>
-      <c r="H8" s="56" t="n"/>
-      <c r="I8" s="55" t="n"/>
-      <c r="J8" s="55" t="n"/>
-      <c r="K8" s="55" t="n"/>
-      <c r="L8" s="55" t="n"/>
-      <c r="M8" s="55" t="n"/>
-      <c r="N8" s="55" t="n"/>
-      <c r="O8" s="55" t="n"/>
-      <c r="P8" s="55" t="n"/>
-      <c r="Q8" s="55" t="n"/>
-      <c r="R8" s="55" t="n"/>
-      <c r="S8" s="55" t="n"/>
-      <c r="T8" s="55" t="n"/>
-      <c r="U8" s="55" t="n"/>
-      <c r="V8" s="55" t="n"/>
-      <c r="W8" s="55" t="n"/>
-      <c r="X8" s="55" t="n"/>
-      <c r="Y8" s="55" t="n"/>
-      <c r="Z8" s="55" t="n"/>
-      <c r="AA8" s="55" t="n"/>
-      <c r="AB8" s="55" t="n"/>
-      <c r="AC8" s="55" t="n"/>
-      <c r="AD8" s="55" t="n"/>
-      <c r="AE8" s="55" t="n"/>
-      <c r="AF8" s="55" t="n"/>
-      <c r="AG8" s="55" t="n"/>
-      <c r="AH8" s="55" t="n"/>
-      <c r="AI8" s="55" t="n"/>
-      <c r="AJ8" s="55" t="n"/>
-      <c r="AK8" s="55" t="n"/>
-      <c r="AL8" s="55" t="n"/>
-      <c r="AM8" s="55" t="n"/>
-      <c r="AN8" s="55" t="n"/>
-      <c r="AO8" s="55" t="n"/>
-      <c r="AP8" s="55" t="n"/>
-      <c r="BG8" s="77" t="n"/>
+      <c r="H8" s="281" t="n"/>
+      <c r="I8" s="282" t="n"/>
+      <c r="J8" s="282" t="n"/>
+      <c r="K8" s="282" t="n"/>
+      <c r="L8" s="282" t="n"/>
+      <c r="M8" s="282" t="n"/>
+      <c r="N8" s="282" t="n"/>
+      <c r="O8" s="282" t="n"/>
+      <c r="P8" s="282" t="n"/>
+      <c r="Q8" s="282" t="n"/>
+      <c r="R8" s="282" t="n"/>
+      <c r="S8" s="282" t="n"/>
+      <c r="T8" s="282" t="n"/>
+      <c r="U8" s="282" t="n"/>
+      <c r="V8" s="282" t="n"/>
+      <c r="W8" s="282" t="n"/>
+      <c r="X8" s="282" t="n"/>
+      <c r="Y8" s="282" t="n"/>
+      <c r="Z8" s="282" t="n"/>
+      <c r="AA8" s="282" t="n"/>
+      <c r="AB8" s="282" t="n"/>
+      <c r="AC8" s="282" t="n"/>
+      <c r="AD8" s="282" t="n"/>
+      <c r="AE8" s="282" t="n"/>
+      <c r="AF8" s="282" t="n"/>
+      <c r="AG8" s="282" t="n"/>
+      <c r="AH8" s="282" t="n"/>
+      <c r="AI8" s="282" t="n"/>
+      <c r="AJ8" s="282" t="n"/>
+      <c r="AK8" s="282" t="n"/>
+      <c r="AL8" s="282" t="n"/>
+      <c r="AM8" s="282" t="n"/>
+      <c r="AN8" s="282" t="n"/>
+      <c r="AO8" s="282" t="n"/>
+      <c r="AP8" s="282" t="n"/>
+      <c r="AQ8" s="283" t="n"/>
+      <c r="AR8" s="283" t="n"/>
+      <c r="AS8" s="283" t="n"/>
+      <c r="AT8" s="283" t="n"/>
+      <c r="AU8" s="283" t="n"/>
+      <c r="AV8" s="283" t="n"/>
+      <c r="AW8" s="283" t="n"/>
+      <c r="AX8" s="283" t="n"/>
+      <c r="AY8" s="283" t="n"/>
+      <c r="AZ8" s="283" t="n"/>
+      <c r="BA8" s="283" t="n"/>
+      <c r="BB8" s="283" t="n"/>
+      <c r="BC8" s="283" t="n"/>
+      <c r="BD8" s="283" t="n"/>
+      <c r="BE8" s="284" t="n"/>
+      <c r="BF8" s="284" t="n"/>
+      <c r="BG8" s="156" t="n"/>
+      <c r="BH8" s="153" t="n"/>
+      <c r="BI8" s="153" t="n"/>
+      <c r="BJ8" s="153" t="n"/>
+      <c r="BK8" s="153" t="n"/>
+      <c r="BL8" s="153" t="n"/>
+      <c r="BM8" s="153" t="n"/>
+      <c r="BN8" s="153" t="n"/>
+      <c r="BO8" s="153" t="n"/>
+      <c r="BP8" s="153" t="n"/>
+      <c r="BQ8" s="153" t="n"/>
+      <c r="BR8" s="153" t="n"/>
+      <c r="BS8" s="153" t="n"/>
+      <c r="BT8" s="153" t="n"/>
+      <c r="BU8" s="153" t="n"/>
+      <c r="BV8" s="153" t="n"/>
+      <c r="BW8" s="153" t="n"/>
+      <c r="BX8" s="153" t="n"/>
+      <c r="BY8" s="153" t="n"/>
+      <c r="BZ8" s="153" t="n"/>
+      <c r="CA8" s="153" t="n"/>
     </row>
-    <row r="9" ht="20" customFormat="1" customHeight="1" s="53" thickBot="1">
-      <c r="A9" s="129" t="n"/>
-      <c r="B9" s="93" t="inlineStr">
+    <row r="9" ht="54" customFormat="1" customHeight="1" s="53" thickBot="1">
+      <c r="A9" s="178" t="n"/>
+      <c r="B9" s="256" t="inlineStr">
         <is>
           <t>Modules</t>
         </is>
       </c>
-      <c r="C9" s="94" t="n">
+      <c r="C9" s="257" t="n">
         <v>1</v>
       </c>
       <c r="D9" s="78" t="n">
@@ -2793,84 +3494,96 @@
       <c r="E9" s="78" t="n">
         <v>45174</v>
       </c>
-      <c r="F9" s="13" t="n"/>
-      <c r="G9" s="3">
+      <c r="F9" s="182" t="n"/>
+      <c r="G9" s="183">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v/>
       </c>
-      <c r="H9" s="135" t="inlineStr">
+      <c r="H9" s="273" t="inlineStr">
         <is>
           <t>CDT taught year - Modules</t>
         </is>
       </c>
-      <c r="I9" s="64" t="n"/>
-      <c r="J9" s="64" t="n"/>
-      <c r="K9" s="64" t="n"/>
-      <c r="L9" s="64" t="n"/>
-      <c r="M9" s="64" t="n"/>
-      <c r="N9" s="64" t="n"/>
-      <c r="O9" s="64" t="n"/>
-      <c r="P9" s="64" t="n"/>
-      <c r="Q9" s="64" t="n"/>
-      <c r="R9" s="64" t="n"/>
-      <c r="S9" s="64" t="n"/>
-      <c r="T9" s="64" t="n"/>
-      <c r="U9" s="64" t="n"/>
-      <c r="V9" s="64" t="n"/>
-      <c r="W9" s="64" t="n"/>
-      <c r="X9" s="64" t="n"/>
-      <c r="Y9" s="64" t="n"/>
-      <c r="Z9" s="64" t="n"/>
-      <c r="AA9" s="64" t="n"/>
-      <c r="AB9" s="64" t="n"/>
-      <c r="AC9" s="64" t="n"/>
-      <c r="AD9" s="64" t="n"/>
-      <c r="AE9" s="64" t="n"/>
-      <c r="AF9" s="64" t="n"/>
-      <c r="AG9" s="64" t="n"/>
-      <c r="AH9" s="64" t="n"/>
-      <c r="AI9" s="64" t="n"/>
-      <c r="AJ9" s="64" t="n"/>
-      <c r="AK9" s="64" t="n"/>
-      <c r="AL9" s="64" t="n"/>
-      <c r="AM9" s="64" t="n"/>
-      <c r="AN9" s="64" t="n"/>
-      <c r="AO9" s="64" t="n"/>
-      <c r="AP9" s="64" t="n"/>
-      <c r="AQ9" s="64" t="n"/>
-      <c r="AR9" s="64" t="n"/>
-      <c r="AS9" s="64" t="n"/>
-      <c r="AT9" s="64" t="n"/>
-      <c r="AU9" s="64" t="n"/>
-      <c r="AV9" s="64" t="n"/>
-      <c r="AW9" s="64" t="n"/>
-      <c r="AX9" s="64" t="n"/>
-      <c r="AY9" s="64" t="n"/>
-      <c r="AZ9" s="64" t="n"/>
-      <c r="BA9" s="64" t="n"/>
-      <c r="BB9" s="64" t="n"/>
-      <c r="BC9" s="64" t="n"/>
-      <c r="BD9" s="64" t="n"/>
-      <c r="BE9" s="59" t="n"/>
-      <c r="BF9" s="35" t="n"/>
-      <c r="BG9" s="79" t="n"/>
-      <c r="BH9" s="59" t="n"/>
-      <c r="BI9" s="35" t="n"/>
-      <c r="BJ9" s="35" t="n"/>
-      <c r="BK9" s="35" t="n"/>
-      <c r="BL9" s="35" t="n"/>
-      <c r="BM9" s="33" t="n"/>
-      <c r="BN9" s="33" t="n"/>
-      <c r="BO9" s="33" t="n"/>
+      <c r="I9" s="282" t="n"/>
+      <c r="J9" s="282" t="n"/>
+      <c r="K9" s="282" t="n"/>
+      <c r="L9" s="282" t="n"/>
+      <c r="M9" s="282" t="n"/>
+      <c r="N9" s="282" t="n"/>
+      <c r="O9" s="282" t="n"/>
+      <c r="P9" s="282" t="n"/>
+      <c r="Q9" s="282" t="n"/>
+      <c r="R9" s="282" t="n"/>
+      <c r="S9" s="282" t="n"/>
+      <c r="T9" s="282" t="n"/>
+      <c r="U9" s="282" t="n"/>
+      <c r="V9" s="282" t="n"/>
+      <c r="W9" s="282" t="n"/>
+      <c r="X9" s="282" t="n"/>
+      <c r="Y9" s="282" t="n"/>
+      <c r="Z9" s="282" t="n"/>
+      <c r="AA9" s="282" t="n"/>
+      <c r="AB9" s="282" t="n"/>
+      <c r="AC9" s="282" t="n"/>
+      <c r="AD9" s="282" t="n"/>
+      <c r="AE9" s="282" t="n"/>
+      <c r="AF9" s="282" t="n"/>
+      <c r="AG9" s="282" t="n"/>
+      <c r="AH9" s="282" t="n"/>
+      <c r="AI9" s="282" t="n"/>
+      <c r="AJ9" s="282" t="n"/>
+      <c r="AK9" s="282" t="n"/>
+      <c r="AL9" s="282" t="n"/>
+      <c r="AM9" s="282" t="n"/>
+      <c r="AN9" s="282" t="n"/>
+      <c r="AO9" s="282" t="n"/>
+      <c r="AP9" s="282" t="n"/>
+      <c r="AQ9" s="282" t="n"/>
+      <c r="AR9" s="282" t="n"/>
+      <c r="AS9" s="282" t="n"/>
+      <c r="AT9" s="282" t="n"/>
+      <c r="AU9" s="282" t="n"/>
+      <c r="AV9" s="282" t="n"/>
+      <c r="AW9" s="282" t="n"/>
+      <c r="AX9" s="282" t="n"/>
+      <c r="AY9" s="282" t="n"/>
+      <c r="AZ9" s="282" t="n"/>
+      <c r="BA9" s="282" t="n"/>
+      <c r="BB9" s="282" t="n"/>
+      <c r="BC9" s="282" t="n"/>
+      <c r="BD9" s="282" t="n"/>
+      <c r="BE9" s="285" t="n"/>
+      <c r="BF9" s="286" t="n"/>
+      <c r="BG9" s="156" t="n"/>
+      <c r="BH9" s="156" t="n"/>
+      <c r="BI9" s="156" t="n"/>
+      <c r="BJ9" s="156" t="n"/>
+      <c r="BK9" s="156" t="n"/>
+      <c r="BL9" s="156" t="n"/>
+      <c r="BM9" s="156" t="n"/>
+      <c r="BN9" s="156" t="n"/>
+      <c r="BO9" s="156" t="n"/>
+      <c r="BP9" s="153" t="n"/>
+      <c r="BQ9" s="153" t="n"/>
+      <c r="BR9" s="153" t="n"/>
+      <c r="BS9" s="153" t="n"/>
+      <c r="BT9" s="153" t="n"/>
+      <c r="BU9" s="153" t="n"/>
+      <c r="BV9" s="153" t="n"/>
+      <c r="BW9" s="153" t="n"/>
+      <c r="BX9" s="153" t="n"/>
+      <c r="BY9" s="153" t="n"/>
+      <c r="BZ9" s="153" t="n"/>
+      <c r="CA9" s="153" t="n"/>
     </row>
-    <row r="10" ht="20" customFormat="1" customHeight="1" s="53" thickBot="1">
-      <c r="A10" s="129" t="n"/>
-      <c r="B10" s="93" t="inlineStr">
+    <row r="10" ht="54" customFormat="1" customHeight="1" s="53" thickBot="1">
+      <c r="A10" s="178" t="n"/>
+      <c r="B10" s="256" t="inlineStr">
         <is>
           <t>Literature</t>
         </is>
       </c>
-      <c r="C10" s="94" t="n">
+      <c r="C10" s="257" t="n">
         <v>1</v>
       </c>
       <c r="D10" s="78" t="n">
@@ -2879,81 +3592,93 @@
       <c r="E10" s="78" t="n">
         <v>44967</v>
       </c>
-      <c r="F10" s="13" t="n"/>
-      <c r="G10" s="3" t="n"/>
-      <c r="H10" s="64" t="n"/>
-      <c r="I10" s="135" t="inlineStr">
+      <c r="F10" s="182" t="n"/>
+      <c r="G10" s="183" t="n"/>
+      <c r="H10" s="282" t="n"/>
+      <c r="I10" s="287" t="inlineStr">
         <is>
           <t>Lit Review</t>
         </is>
       </c>
-      <c r="J10" s="64" t="n"/>
-      <c r="K10" s="64" t="n"/>
-      <c r="L10" s="64" t="n"/>
-      <c r="M10" s="64" t="n"/>
-      <c r="N10" s="64" t="n"/>
-      <c r="O10" s="64" t="n"/>
-      <c r="P10" s="64" t="n"/>
-      <c r="Q10" s="64" t="n"/>
-      <c r="R10" s="64" t="n"/>
-      <c r="S10" s="64" t="n"/>
-      <c r="T10" s="64" t="n"/>
-      <c r="U10" s="64" t="n"/>
-      <c r="V10" s="64" t="n"/>
-      <c r="W10" s="64" t="n"/>
-      <c r="X10" s="64" t="n"/>
-      <c r="Y10" s="64" t="n"/>
-      <c r="Z10" s="64" t="n"/>
-      <c r="AA10" s="64" t="n"/>
-      <c r="AB10" s="64" t="n"/>
-      <c r="AC10" s="64" t="n"/>
-      <c r="AD10" s="64" t="n"/>
-      <c r="AE10" s="64" t="n"/>
-      <c r="AF10" s="64" t="n"/>
-      <c r="AG10" s="64" t="n"/>
-      <c r="AH10" s="64" t="n"/>
-      <c r="AI10" s="64" t="n"/>
-      <c r="AJ10" s="64" t="n"/>
-      <c r="AK10" s="64" t="n"/>
-      <c r="AL10" s="64" t="n"/>
-      <c r="AM10" s="64" t="n"/>
-      <c r="AN10" s="64" t="n"/>
-      <c r="AO10" s="64" t="n"/>
-      <c r="AP10" s="64" t="n"/>
-      <c r="AQ10" s="64" t="n"/>
-      <c r="AR10" s="64" t="n"/>
-      <c r="AS10" s="64" t="n"/>
-      <c r="AT10" s="64" t="n"/>
-      <c r="AU10" s="64" t="n"/>
-      <c r="AV10" s="64" t="n"/>
-      <c r="AW10" s="64" t="n"/>
-      <c r="AX10" s="64" t="n"/>
-      <c r="AY10" s="64" t="n"/>
-      <c r="AZ10" s="64" t="n"/>
-      <c r="BA10" s="64" t="n"/>
-      <c r="BB10" s="64" t="n"/>
-      <c r="BC10" s="64" t="n"/>
-      <c r="BD10" s="64" t="n"/>
-      <c r="BE10" s="59" t="n"/>
-      <c r="BF10" s="35" t="n"/>
-      <c r="BG10" s="79" t="n"/>
-      <c r="BH10" s="59" t="n"/>
-      <c r="BI10" s="35" t="n"/>
-      <c r="BJ10" s="35" t="n"/>
-      <c r="BK10" s="35" t="n"/>
-      <c r="BL10" s="35" t="n"/>
-      <c r="BM10" s="33" t="n"/>
-      <c r="BN10" s="33" t="n"/>
-      <c r="BO10" s="33" t="n"/>
+      <c r="J10" s="282" t="n"/>
+      <c r="K10" s="282" t="n"/>
+      <c r="L10" s="282" t="n"/>
+      <c r="M10" s="282" t="n"/>
+      <c r="N10" s="282" t="n"/>
+      <c r="O10" s="282" t="n"/>
+      <c r="P10" s="282" t="n"/>
+      <c r="Q10" s="282" t="n"/>
+      <c r="R10" s="282" t="n"/>
+      <c r="S10" s="282" t="n"/>
+      <c r="T10" s="282" t="n"/>
+      <c r="U10" s="282" t="n"/>
+      <c r="V10" s="282" t="n"/>
+      <c r="W10" s="282" t="n"/>
+      <c r="X10" s="282" t="n"/>
+      <c r="Y10" s="282" t="n"/>
+      <c r="Z10" s="282" t="n"/>
+      <c r="AA10" s="282" t="n"/>
+      <c r="AB10" s="282" t="n"/>
+      <c r="AC10" s="282" t="n"/>
+      <c r="AD10" s="282" t="n"/>
+      <c r="AE10" s="282" t="n"/>
+      <c r="AF10" s="282" t="n"/>
+      <c r="AG10" s="282" t="n"/>
+      <c r="AH10" s="282" t="n"/>
+      <c r="AI10" s="282" t="n"/>
+      <c r="AJ10" s="282" t="n"/>
+      <c r="AK10" s="282" t="n"/>
+      <c r="AL10" s="282" t="n"/>
+      <c r="AM10" s="282" t="n"/>
+      <c r="AN10" s="282" t="n"/>
+      <c r="AO10" s="282" t="n"/>
+      <c r="AP10" s="282" t="n"/>
+      <c r="AQ10" s="282" t="n"/>
+      <c r="AR10" s="282" t="n"/>
+      <c r="AS10" s="282" t="n"/>
+      <c r="AT10" s="282" t="n"/>
+      <c r="AU10" s="282" t="n"/>
+      <c r="AV10" s="282" t="n"/>
+      <c r="AW10" s="282" t="n"/>
+      <c r="AX10" s="282" t="n"/>
+      <c r="AY10" s="282" t="n"/>
+      <c r="AZ10" s="282" t="n"/>
+      <c r="BA10" s="282" t="n"/>
+      <c r="BB10" s="282" t="n"/>
+      <c r="BC10" s="282" t="n"/>
+      <c r="BD10" s="282" t="n"/>
+      <c r="BE10" s="285" t="n"/>
+      <c r="BF10" s="286" t="n"/>
+      <c r="BG10" s="156" t="n"/>
+      <c r="BH10" s="156" t="n"/>
+      <c r="BI10" s="156" t="n"/>
+      <c r="BJ10" s="156" t="n"/>
+      <c r="BK10" s="156" t="n"/>
+      <c r="BL10" s="156" t="n"/>
+      <c r="BM10" s="156" t="n"/>
+      <c r="BN10" s="156" t="n"/>
+      <c r="BO10" s="156" t="n"/>
+      <c r="BP10" s="153" t="n"/>
+      <c r="BQ10" s="153" t="n"/>
+      <c r="BR10" s="153" t="n"/>
+      <c r="BS10" s="153" t="n"/>
+      <c r="BT10" s="153" t="n"/>
+      <c r="BU10" s="153" t="n"/>
+      <c r="BV10" s="153" t="n"/>
+      <c r="BW10" s="153" t="n"/>
+      <c r="BX10" s="153" t="n"/>
+      <c r="BY10" s="153" t="n"/>
+      <c r="BZ10" s="153" t="n"/>
+      <c r="CA10" s="153" t="n"/>
     </row>
-    <row r="11" ht="20" customFormat="1" customHeight="1" s="53" thickBot="1">
-      <c r="A11" s="129" t="n"/>
-      <c r="B11" s="93" t="inlineStr">
+    <row r="11" ht="54" customFormat="1" customHeight="1" s="53" thickBot="1">
+      <c r="A11" s="178" t="n"/>
+      <c r="B11" s="256" t="inlineStr">
         <is>
           <t>Systematic review</t>
         </is>
       </c>
-      <c r="C11" s="94" t="n">
+      <c r="C11" s="257" t="n">
         <v>1</v>
       </c>
       <c r="D11" s="78" t="n">
@@ -2962,84 +3687,96 @@
       <c r="E11" s="78" t="n">
         <v>45058</v>
       </c>
-      <c r="F11" s="13" t="n"/>
-      <c r="G11" s="3">
+      <c r="F11" s="182" t="n"/>
+      <c r="G11" s="183">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v/>
       </c>
-      <c r="H11" s="64" t="n"/>
-      <c r="I11" s="64" t="n"/>
-      <c r="J11" s="135" t="inlineStr">
+      <c r="H11" s="282" t="n"/>
+      <c r="I11" s="282" t="n"/>
+      <c r="J11" s="287" t="inlineStr">
         <is>
           <t>Sytematic Review</t>
         </is>
       </c>
-      <c r="K11" s="64" t="n"/>
-      <c r="L11" s="64" t="n"/>
-      <c r="M11" s="64" t="n"/>
-      <c r="N11" s="64" t="n"/>
-      <c r="O11" s="64" t="n"/>
-      <c r="P11" s="64" t="n"/>
-      <c r="Q11" s="64" t="n"/>
-      <c r="R11" s="64" t="n"/>
-      <c r="S11" s="64" t="n"/>
-      <c r="T11" s="64" t="n"/>
-      <c r="U11" s="64" t="n"/>
-      <c r="V11" s="64" t="n"/>
-      <c r="W11" s="64" t="n"/>
-      <c r="X11" s="64" t="n"/>
-      <c r="Y11" s="64" t="n"/>
-      <c r="Z11" s="64" t="n"/>
-      <c r="AA11" s="64" t="n"/>
-      <c r="AB11" s="64" t="n"/>
-      <c r="AC11" s="64" t="n"/>
-      <c r="AD11" s="64" t="n"/>
-      <c r="AE11" s="64" t="n"/>
-      <c r="AF11" s="64" t="n"/>
-      <c r="AG11" s="64" t="n"/>
-      <c r="AH11" s="64" t="n"/>
-      <c r="AI11" s="64" t="n"/>
-      <c r="AJ11" s="64" t="n"/>
-      <c r="AK11" s="64" t="n"/>
-      <c r="AL11" s="64" t="n"/>
-      <c r="AM11" s="64" t="n"/>
-      <c r="AN11" s="64" t="n"/>
-      <c r="AO11" s="64" t="n"/>
-      <c r="AP11" s="64" t="n"/>
-      <c r="AQ11" s="64" t="n"/>
-      <c r="AR11" s="64" t="n"/>
-      <c r="AS11" s="64" t="n"/>
-      <c r="AT11" s="64" t="n"/>
-      <c r="AU11" s="64" t="n"/>
-      <c r="AV11" s="64" t="n"/>
-      <c r="AW11" s="64" t="n"/>
-      <c r="AX11" s="64" t="n"/>
-      <c r="AY11" s="64" t="n"/>
-      <c r="AZ11" s="64" t="n"/>
-      <c r="BA11" s="64" t="n"/>
-      <c r="BB11" s="64" t="n"/>
-      <c r="BC11" s="64" t="n"/>
-      <c r="BD11" s="64" t="n"/>
-      <c r="BE11" s="60" t="n"/>
-      <c r="BF11" s="33" t="n"/>
-      <c r="BG11" s="80" t="n"/>
-      <c r="BH11" s="60" t="n"/>
-      <c r="BI11" s="33" t="n"/>
-      <c r="BJ11" s="33" t="n"/>
-      <c r="BK11" s="33" t="n"/>
-      <c r="BL11" s="33" t="n"/>
-      <c r="BM11" s="33" t="n"/>
-      <c r="BN11" s="33" t="n"/>
-      <c r="BO11" s="33" t="n"/>
+      <c r="K11" s="282" t="n"/>
+      <c r="L11" s="282" t="n"/>
+      <c r="M11" s="282" t="n"/>
+      <c r="N11" s="282" t="n"/>
+      <c r="O11" s="282" t="n"/>
+      <c r="P11" s="282" t="n"/>
+      <c r="Q11" s="282" t="n"/>
+      <c r="R11" s="282" t="n"/>
+      <c r="S11" s="282" t="n"/>
+      <c r="T11" s="282" t="n"/>
+      <c r="U11" s="282" t="n"/>
+      <c r="V11" s="282" t="n"/>
+      <c r="W11" s="282" t="n"/>
+      <c r="X11" s="282" t="n"/>
+      <c r="Y11" s="282" t="n"/>
+      <c r="Z11" s="282" t="n"/>
+      <c r="AA11" s="282" t="n"/>
+      <c r="AB11" s="282" t="n"/>
+      <c r="AC11" s="282" t="n"/>
+      <c r="AD11" s="282" t="n"/>
+      <c r="AE11" s="282" t="n"/>
+      <c r="AF11" s="282" t="n"/>
+      <c r="AG11" s="282" t="n"/>
+      <c r="AH11" s="282" t="n"/>
+      <c r="AI11" s="282" t="n"/>
+      <c r="AJ11" s="282" t="n"/>
+      <c r="AK11" s="282" t="n"/>
+      <c r="AL11" s="282" t="n"/>
+      <c r="AM11" s="282" t="n"/>
+      <c r="AN11" s="282" t="n"/>
+      <c r="AO11" s="282" t="n"/>
+      <c r="AP11" s="282" t="n"/>
+      <c r="AQ11" s="282" t="n"/>
+      <c r="AR11" s="282" t="n"/>
+      <c r="AS11" s="282" t="n"/>
+      <c r="AT11" s="282" t="n"/>
+      <c r="AU11" s="282" t="n"/>
+      <c r="AV11" s="282" t="n"/>
+      <c r="AW11" s="282" t="n"/>
+      <c r="AX11" s="282" t="n"/>
+      <c r="AY11" s="282" t="n"/>
+      <c r="AZ11" s="282" t="n"/>
+      <c r="BA11" s="282" t="n"/>
+      <c r="BB11" s="282" t="n"/>
+      <c r="BC11" s="282" t="n"/>
+      <c r="BD11" s="282" t="n"/>
+      <c r="BE11" s="288" t="n"/>
+      <c r="BF11" s="289" t="n"/>
+      <c r="BG11" s="156" t="n"/>
+      <c r="BH11" s="156" t="n"/>
+      <c r="BI11" s="156" t="n"/>
+      <c r="BJ11" s="156" t="n"/>
+      <c r="BK11" s="156" t="n"/>
+      <c r="BL11" s="156" t="n"/>
+      <c r="BM11" s="156" t="n"/>
+      <c r="BN11" s="156" t="n"/>
+      <c r="BO11" s="156" t="n"/>
+      <c r="BP11" s="153" t="n"/>
+      <c r="BQ11" s="153" t="n"/>
+      <c r="BR11" s="153" t="n"/>
+      <c r="BS11" s="153" t="n"/>
+      <c r="BT11" s="153" t="n"/>
+      <c r="BU11" s="153" t="n"/>
+      <c r="BV11" s="153" t="n"/>
+      <c r="BW11" s="153" t="n"/>
+      <c r="BX11" s="153" t="n"/>
+      <c r="BY11" s="153" t="n"/>
+      <c r="BZ11" s="153" t="n"/>
+      <c r="CA11" s="153" t="n"/>
     </row>
-    <row r="12" ht="20" customFormat="1" customHeight="1" s="53" thickBot="1">
-      <c r="A12" s="130" t="n"/>
-      <c r="B12" s="93" t="inlineStr">
+    <row r="12" ht="54" customFormat="1" customHeight="1" s="53" thickBot="1">
+      <c r="A12" s="197" t="n"/>
+      <c r="B12" s="256" t="inlineStr">
         <is>
           <t>Final project</t>
         </is>
       </c>
-      <c r="C12" s="94" t="n">
+      <c r="C12" s="257" t="n">
         <v>1</v>
       </c>
       <c r="D12" s="78" t="n">
@@ -3048,84 +3785,96 @@
       <c r="E12" s="78" t="n">
         <v>45108</v>
       </c>
-      <c r="F12" s="13" t="n"/>
-      <c r="G12" s="3">
+      <c r="F12" s="182" t="n"/>
+      <c r="G12" s="183">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v/>
       </c>
-      <c r="H12" s="64" t="n"/>
-      <c r="I12" s="64" t="n"/>
-      <c r="J12" s="64" t="n"/>
-      <c r="K12" s="64" t="n"/>
-      <c r="L12" s="135" t="inlineStr">
+      <c r="H12" s="282" t="n"/>
+      <c r="I12" s="282" t="n"/>
+      <c r="J12" s="282" t="n"/>
+      <c r="K12" s="282" t="n"/>
+      <c r="L12" s="287" t="inlineStr">
         <is>
           <t>Final project</t>
         </is>
       </c>
-      <c r="M12" s="64" t="n"/>
-      <c r="N12" s="64" t="n"/>
-      <c r="O12" s="64" t="n"/>
-      <c r="P12" s="64" t="n"/>
-      <c r="Q12" s="64" t="n"/>
-      <c r="R12" s="64" t="n"/>
-      <c r="S12" s="64" t="n"/>
-      <c r="T12" s="64" t="n"/>
-      <c r="U12" s="64" t="n"/>
-      <c r="V12" s="64" t="n"/>
-      <c r="W12" s="64" t="n"/>
-      <c r="X12" s="64" t="n"/>
-      <c r="Y12" s="64" t="n"/>
-      <c r="Z12" s="64" t="n"/>
-      <c r="AA12" s="64" t="n"/>
-      <c r="AB12" s="64" t="n"/>
-      <c r="AC12" s="64" t="n"/>
-      <c r="AD12" s="64" t="n"/>
-      <c r="AE12" s="64" t="n"/>
-      <c r="AF12" s="64" t="n"/>
-      <c r="AG12" s="64" t="n"/>
-      <c r="AH12" s="64" t="n"/>
-      <c r="AI12" s="64" t="n"/>
-      <c r="AJ12" s="64" t="n"/>
-      <c r="AK12" s="64" t="n"/>
-      <c r="AL12" s="64" t="n"/>
-      <c r="AM12" s="64" t="n"/>
-      <c r="AN12" s="64" t="n"/>
-      <c r="AO12" s="64" t="n"/>
-      <c r="AP12" s="64" t="n"/>
-      <c r="AQ12" s="64" t="n"/>
-      <c r="AR12" s="64" t="n"/>
-      <c r="AS12" s="64" t="n"/>
-      <c r="AT12" s="64" t="n"/>
-      <c r="AU12" s="64" t="n"/>
-      <c r="AV12" s="64" t="n"/>
-      <c r="AW12" s="64" t="n"/>
-      <c r="AX12" s="64" t="n"/>
-      <c r="AY12" s="64" t="n"/>
-      <c r="AZ12" s="64" t="n"/>
-      <c r="BA12" s="64" t="n"/>
-      <c r="BB12" s="64" t="n"/>
-      <c r="BC12" s="64" t="n"/>
-      <c r="BD12" s="64" t="n"/>
-      <c r="BE12" s="60" t="n"/>
-      <c r="BF12" s="33" t="n"/>
-      <c r="BG12" s="80" t="n"/>
-      <c r="BH12" s="60" t="n"/>
-      <c r="BI12" s="33" t="n"/>
-      <c r="BJ12" s="33" t="n"/>
-      <c r="BK12" s="33" t="n"/>
-      <c r="BL12" s="33" t="n"/>
-      <c r="BM12" s="33" t="n"/>
-      <c r="BN12" s="33" t="n"/>
-      <c r="BO12" s="33" t="n"/>
+      <c r="M12" s="282" t="n"/>
+      <c r="N12" s="282" t="n"/>
+      <c r="O12" s="282" t="n"/>
+      <c r="P12" s="282" t="n"/>
+      <c r="Q12" s="282" t="n"/>
+      <c r="R12" s="282" t="n"/>
+      <c r="S12" s="282" t="n"/>
+      <c r="T12" s="282" t="n"/>
+      <c r="U12" s="282" t="n"/>
+      <c r="V12" s="282" t="n"/>
+      <c r="W12" s="282" t="n"/>
+      <c r="X12" s="282" t="n"/>
+      <c r="Y12" s="282" t="n"/>
+      <c r="Z12" s="282" t="n"/>
+      <c r="AA12" s="282" t="n"/>
+      <c r="AB12" s="282" t="n"/>
+      <c r="AC12" s="282" t="n"/>
+      <c r="AD12" s="282" t="n"/>
+      <c r="AE12" s="282" t="n"/>
+      <c r="AF12" s="282" t="n"/>
+      <c r="AG12" s="282" t="n"/>
+      <c r="AH12" s="282" t="n"/>
+      <c r="AI12" s="282" t="n"/>
+      <c r="AJ12" s="282" t="n"/>
+      <c r="AK12" s="282" t="n"/>
+      <c r="AL12" s="282" t="n"/>
+      <c r="AM12" s="282" t="n"/>
+      <c r="AN12" s="282" t="n"/>
+      <c r="AO12" s="282" t="n"/>
+      <c r="AP12" s="282" t="n"/>
+      <c r="AQ12" s="282" t="n"/>
+      <c r="AR12" s="282" t="n"/>
+      <c r="AS12" s="282" t="n"/>
+      <c r="AT12" s="282" t="n"/>
+      <c r="AU12" s="282" t="n"/>
+      <c r="AV12" s="282" t="n"/>
+      <c r="AW12" s="282" t="n"/>
+      <c r="AX12" s="282" t="n"/>
+      <c r="AY12" s="282" t="n"/>
+      <c r="AZ12" s="282" t="n"/>
+      <c r="BA12" s="282" t="n"/>
+      <c r="BB12" s="282" t="n"/>
+      <c r="BC12" s="282" t="n"/>
+      <c r="BD12" s="282" t="n"/>
+      <c r="BE12" s="288" t="n"/>
+      <c r="BF12" s="289" t="n"/>
+      <c r="BG12" s="156" t="n"/>
+      <c r="BH12" s="156" t="n"/>
+      <c r="BI12" s="156" t="n"/>
+      <c r="BJ12" s="156" t="n"/>
+      <c r="BK12" s="156" t="n"/>
+      <c r="BL12" s="156" t="n"/>
+      <c r="BM12" s="156" t="n"/>
+      <c r="BN12" s="156" t="n"/>
+      <c r="BO12" s="156" t="n"/>
+      <c r="BP12" s="153" t="n"/>
+      <c r="BQ12" s="153" t="n"/>
+      <c r="BR12" s="153" t="n"/>
+      <c r="BS12" s="153" t="n"/>
+      <c r="BT12" s="153" t="n"/>
+      <c r="BU12" s="153" t="n"/>
+      <c r="BV12" s="153" t="n"/>
+      <c r="BW12" s="153" t="n"/>
+      <c r="BX12" s="153" t="n"/>
+      <c r="BY12" s="153" t="n"/>
+      <c r="BZ12" s="153" t="n"/>
+      <c r="CA12" s="153" t="n"/>
     </row>
-    <row r="13" ht="20" customFormat="1" customHeight="1" s="53" thickBot="1">
-      <c r="A13" s="130" t="n"/>
-      <c r="B13" s="93" t="inlineStr">
+    <row r="13" ht="54" customFormat="1" customHeight="1" s="53" thickBot="1">
+      <c r="A13" s="197" t="n"/>
+      <c r="B13" s="256" t="inlineStr">
         <is>
           <t>Research design</t>
         </is>
       </c>
-      <c r="C13" s="94" t="n">
+      <c r="C13" s="257" t="n">
         <v>1</v>
       </c>
       <c r="D13" s="78" t="n">
@@ -3134,81 +3883,93 @@
       <c r="E13" s="78" t="n">
         <v>45293</v>
       </c>
-      <c r="F13" s="13" t="n"/>
-      <c r="G13" s="62" t="n"/>
-      <c r="H13" s="64" t="n"/>
-      <c r="I13" s="64" t="n"/>
-      <c r="J13" s="64" t="n"/>
-      <c r="K13" s="64" t="n"/>
-      <c r="L13" s="64" t="n"/>
-      <c r="M13" s="64" t="n"/>
-      <c r="N13" s="64" t="n"/>
-      <c r="O13" s="64" t="n"/>
-      <c r="P13" s="64" t="n"/>
-      <c r="Q13" s="64" t="n"/>
-      <c r="R13" s="64" t="n"/>
-      <c r="S13" s="64" t="n"/>
-      <c r="T13" s="136" t="inlineStr">
+      <c r="F13" s="182" t="n"/>
+      <c r="G13" s="198" t="n"/>
+      <c r="H13" s="282" t="n"/>
+      <c r="I13" s="282" t="n"/>
+      <c r="J13" s="282" t="n"/>
+      <c r="K13" s="282" t="n"/>
+      <c r="L13" s="282" t="n"/>
+      <c r="M13" s="282" t="n"/>
+      <c r="N13" s="282" t="n"/>
+      <c r="O13" s="282" t="n"/>
+      <c r="P13" s="282" t="n"/>
+      <c r="Q13" s="282" t="n"/>
+      <c r="R13" s="282" t="n"/>
+      <c r="S13" s="282" t="n"/>
+      <c r="T13" s="287" t="inlineStr">
         <is>
           <t>R. Design</t>
         </is>
       </c>
-      <c r="U13" s="137" t="n"/>
-      <c r="V13" s="137" t="n"/>
-      <c r="W13" s="138" t="n"/>
-      <c r="X13" s="64" t="n"/>
-      <c r="Y13" s="64" t="n"/>
-      <c r="Z13" s="64" t="n"/>
-      <c r="AA13" s="64" t="n"/>
-      <c r="AB13" s="64" t="n"/>
-      <c r="AC13" s="64" t="n"/>
-      <c r="AD13" s="64" t="n"/>
-      <c r="AE13" s="64" t="n"/>
-      <c r="AF13" s="64" t="n"/>
-      <c r="AG13" s="64" t="n"/>
-      <c r="AH13" s="64" t="n"/>
-      <c r="AI13" s="64" t="n"/>
-      <c r="AJ13" s="64" t="n"/>
-      <c r="AK13" s="64" t="n"/>
-      <c r="AL13" s="64" t="n"/>
-      <c r="AM13" s="64" t="n"/>
-      <c r="AN13" s="64" t="n"/>
-      <c r="AO13" s="64" t="n"/>
-      <c r="AP13" s="64" t="n"/>
-      <c r="AQ13" s="64" t="n"/>
-      <c r="AR13" s="64" t="n"/>
-      <c r="AS13" s="64" t="n"/>
-      <c r="AT13" s="64" t="n"/>
-      <c r="AU13" s="64" t="n"/>
-      <c r="AV13" s="64" t="n"/>
-      <c r="AW13" s="64" t="n"/>
-      <c r="AX13" s="64" t="n"/>
-      <c r="AY13" s="64" t="n"/>
-      <c r="AZ13" s="64" t="n"/>
-      <c r="BA13" s="64" t="n"/>
-      <c r="BB13" s="64" t="n"/>
-      <c r="BC13" s="64" t="n"/>
-      <c r="BD13" s="64" t="n"/>
-      <c r="BE13" s="60" t="n"/>
-      <c r="BF13" s="33" t="n"/>
-      <c r="BG13" s="80" t="n"/>
-      <c r="BH13" s="60" t="n"/>
-      <c r="BI13" s="33" t="n"/>
-      <c r="BJ13" s="33" t="n"/>
-      <c r="BK13" s="33" t="n"/>
-      <c r="BL13" s="33" t="n"/>
-      <c r="BM13" s="33" t="n"/>
-      <c r="BN13" s="33" t="n"/>
-      <c r="BO13" s="33" t="n"/>
+      <c r="U13" s="282" t="n"/>
+      <c r="V13" s="282" t="n"/>
+      <c r="W13" s="282" t="n"/>
+      <c r="X13" s="282" t="n"/>
+      <c r="Y13" s="282" t="n"/>
+      <c r="Z13" s="282" t="n"/>
+      <c r="AA13" s="282" t="n"/>
+      <c r="AB13" s="282" t="n"/>
+      <c r="AC13" s="282" t="n"/>
+      <c r="AD13" s="282" t="n"/>
+      <c r="AE13" s="282" t="n"/>
+      <c r="AF13" s="282" t="n"/>
+      <c r="AG13" s="282" t="n"/>
+      <c r="AH13" s="282" t="n"/>
+      <c r="AI13" s="282" t="n"/>
+      <c r="AJ13" s="282" t="n"/>
+      <c r="AK13" s="282" t="n"/>
+      <c r="AL13" s="282" t="n"/>
+      <c r="AM13" s="282" t="n"/>
+      <c r="AN13" s="282" t="n"/>
+      <c r="AO13" s="282" t="n"/>
+      <c r="AP13" s="282" t="n"/>
+      <c r="AQ13" s="282" t="n"/>
+      <c r="AR13" s="282" t="n"/>
+      <c r="AS13" s="282" t="n"/>
+      <c r="AT13" s="282" t="n"/>
+      <c r="AU13" s="282" t="n"/>
+      <c r="AV13" s="282" t="n"/>
+      <c r="AW13" s="282" t="n"/>
+      <c r="AX13" s="282" t="n"/>
+      <c r="AY13" s="282" t="n"/>
+      <c r="AZ13" s="282" t="n"/>
+      <c r="BA13" s="282" t="n"/>
+      <c r="BB13" s="282" t="n"/>
+      <c r="BC13" s="282" t="n"/>
+      <c r="BD13" s="282" t="n"/>
+      <c r="BE13" s="288" t="n"/>
+      <c r="BF13" s="289" t="n"/>
+      <c r="BG13" s="156" t="n"/>
+      <c r="BH13" s="156" t="n"/>
+      <c r="BI13" s="156" t="n"/>
+      <c r="BJ13" s="156" t="n"/>
+      <c r="BK13" s="156" t="n"/>
+      <c r="BL13" s="156" t="n"/>
+      <c r="BM13" s="156" t="n"/>
+      <c r="BN13" s="156" t="n"/>
+      <c r="BO13" s="156" t="n"/>
+      <c r="BP13" s="153" t="n"/>
+      <c r="BQ13" s="153" t="n"/>
+      <c r="BR13" s="153" t="n"/>
+      <c r="BS13" s="153" t="n"/>
+      <c r="BT13" s="153" t="n"/>
+      <c r="BU13" s="153" t="n"/>
+      <c r="BV13" s="153" t="n"/>
+      <c r="BW13" s="153" t="n"/>
+      <c r="BX13" s="153" t="n"/>
+      <c r="BY13" s="153" t="n"/>
+      <c r="BZ13" s="153" t="n"/>
+      <c r="CA13" s="153" t="n"/>
     </row>
-    <row r="14" ht="20" customFormat="1" customHeight="1" s="53" thickBot="1">
-      <c r="A14" s="130" t="n"/>
-      <c r="B14" s="93" t="inlineStr">
+    <row r="14" ht="54" customFormat="1" customHeight="1" s="53" thickBot="1">
+      <c r="A14" s="197" t="n"/>
+      <c r="B14" s="256" t="inlineStr">
         <is>
           <t>Upgrade Report</t>
         </is>
       </c>
-      <c r="C14" s="94" t="n">
+      <c r="C14" s="257" t="n">
         <v>1</v>
       </c>
       <c r="D14" s="78" t="n">
@@ -3217,341 +3978,476 @@
       <c r="E14" s="78" t="n">
         <v>45962</v>
       </c>
-      <c r="F14" s="13" t="n"/>
-      <c r="G14" s="62">
+      <c r="F14" s="182" t="n"/>
+      <c r="G14" s="198">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v/>
       </c>
-      <c r="H14" s="68" t="n"/>
-      <c r="I14" s="68" t="n"/>
-      <c r="J14" s="68" t="n"/>
-      <c r="K14" s="68" t="n"/>
-      <c r="L14" s="68" t="n"/>
-      <c r="M14" s="68" t="n"/>
-      <c r="N14" s="68" t="n"/>
-      <c r="O14" s="68" t="n"/>
-      <c r="P14" s="68" t="n"/>
-      <c r="Q14" s="68" t="n"/>
-      <c r="R14" s="68" t="n"/>
-      <c r="S14" s="68" t="n"/>
-      <c r="T14" s="68" t="n"/>
-      <c r="U14" s="68" t="n"/>
-      <c r="V14" s="68" t="n"/>
-      <c r="W14" s="68" t="n"/>
-      <c r="X14" s="139" t="inlineStr">
+      <c r="H14" s="282" t="n"/>
+      <c r="I14" s="282" t="n"/>
+      <c r="J14" s="282" t="n"/>
+      <c r="K14" s="282" t="n"/>
+      <c r="L14" s="282" t="n"/>
+      <c r="M14" s="282" t="n"/>
+      <c r="N14" s="282" t="n"/>
+      <c r="O14" s="282" t="n"/>
+      <c r="P14" s="282" t="n"/>
+      <c r="Q14" s="282" t="n"/>
+      <c r="R14" s="282" t="n"/>
+      <c r="S14" s="282" t="n"/>
+      <c r="T14" s="282" t="n"/>
+      <c r="U14" s="282" t="n"/>
+      <c r="V14" s="282" t="n"/>
+      <c r="W14" s="282" t="n"/>
+      <c r="X14" s="287" t="inlineStr">
         <is>
           <t>This report</t>
         </is>
       </c>
-      <c r="Y14" s="68" t="n"/>
-      <c r="Z14" s="68" t="n"/>
-      <c r="AA14" s="68" t="n"/>
-      <c r="AB14" s="68" t="n"/>
-      <c r="AC14" s="68" t="n"/>
-      <c r="AD14" s="68" t="n"/>
-      <c r="AE14" s="68" t="n"/>
-      <c r="AF14" s="68" t="n"/>
-      <c r="AG14" s="68" t="n"/>
-      <c r="AH14" s="68" t="n"/>
-      <c r="AI14" s="68" t="n"/>
-      <c r="AJ14" s="68" t="n"/>
-      <c r="AK14" s="68" t="n"/>
-      <c r="AL14" s="68" t="n"/>
-      <c r="AM14" s="68" t="n"/>
-      <c r="AN14" s="68" t="n"/>
-      <c r="AO14" s="68" t="n"/>
-      <c r="AP14" s="68" t="n"/>
-      <c r="AQ14" s="68" t="n"/>
-      <c r="AR14" s="68" t="n"/>
-      <c r="AS14" s="68" t="n"/>
-      <c r="AT14" s="68" t="n"/>
-      <c r="AU14" s="68" t="n"/>
-      <c r="AV14" s="68" t="n"/>
-      <c r="AW14" s="68" t="n"/>
-      <c r="AX14" s="68" t="n"/>
-      <c r="AY14" s="68" t="n"/>
-      <c r="AZ14" s="68" t="n"/>
-      <c r="BA14" s="68" t="n"/>
-      <c r="BB14" s="68" t="n"/>
-      <c r="BC14" s="68" t="n"/>
-      <c r="BD14" s="68" t="n"/>
-      <c r="BE14" s="60" t="n"/>
-      <c r="BF14" s="33" t="n"/>
-      <c r="BG14" s="80" t="n"/>
-      <c r="BH14" s="60" t="n"/>
-      <c r="BI14" s="33" t="n"/>
-      <c r="BJ14" s="33" t="n"/>
-      <c r="BK14" s="33" t="n"/>
-      <c r="BL14" s="33" t="n"/>
-      <c r="BM14" s="33" t="n"/>
-      <c r="BN14" s="33" t="n"/>
-      <c r="BO14" s="33" t="n"/>
+      <c r="Y14" s="282" t="n"/>
+      <c r="Z14" s="282" t="n"/>
+      <c r="AA14" s="282" t="n"/>
+      <c r="AB14" s="282" t="n"/>
+      <c r="AC14" s="282" t="n"/>
+      <c r="AD14" s="282" t="n"/>
+      <c r="AE14" s="282" t="n"/>
+      <c r="AF14" s="282" t="n"/>
+      <c r="AG14" s="282" t="n"/>
+      <c r="AH14" s="282" t="n"/>
+      <c r="AI14" s="282" t="n"/>
+      <c r="AJ14" s="282" t="n"/>
+      <c r="AK14" s="282" t="n"/>
+      <c r="AL14" s="282" t="n"/>
+      <c r="AM14" s="282" t="n"/>
+      <c r="AN14" s="282" t="n"/>
+      <c r="AO14" s="282" t="n"/>
+      <c r="AP14" s="282" t="n"/>
+      <c r="AQ14" s="282" t="n"/>
+      <c r="AR14" s="282" t="n"/>
+      <c r="AS14" s="282" t="n"/>
+      <c r="AT14" s="282" t="n"/>
+      <c r="AU14" s="282" t="n"/>
+      <c r="AV14" s="282" t="n"/>
+      <c r="AW14" s="282" t="n"/>
+      <c r="AX14" s="282" t="n"/>
+      <c r="AY14" s="282" t="n"/>
+      <c r="AZ14" s="282" t="n"/>
+      <c r="BA14" s="282" t="n"/>
+      <c r="BB14" s="282" t="n"/>
+      <c r="BC14" s="282" t="n"/>
+      <c r="BD14" s="282" t="n"/>
+      <c r="BE14" s="288" t="n"/>
+      <c r="BF14" s="289" t="n"/>
+      <c r="BG14" s="156" t="n"/>
+      <c r="BH14" s="156" t="n"/>
+      <c r="BI14" s="156" t="n"/>
+      <c r="BJ14" s="156" t="n"/>
+      <c r="BK14" s="156" t="n"/>
+      <c r="BL14" s="156" t="n"/>
+      <c r="BM14" s="156" t="n"/>
+      <c r="BN14" s="156" t="n"/>
+      <c r="BO14" s="156" t="n"/>
+      <c r="BP14" s="153" t="n"/>
+      <c r="BQ14" s="153" t="n"/>
+      <c r="BR14" s="153" t="n"/>
+      <c r="BS14" s="153" t="n"/>
+      <c r="BT14" s="153" t="n"/>
+      <c r="BU14" s="153" t="n"/>
+      <c r="BV14" s="153" t="n"/>
+      <c r="BW14" s="153" t="n"/>
+      <c r="BX14" s="153" t="n"/>
+      <c r="BY14" s="153" t="n"/>
+      <c r="BZ14" s="153" t="n"/>
+      <c r="CA14" s="153" t="n"/>
     </row>
-    <row r="15" ht="20" customFormat="1" customHeight="1" s="53" thickBot="1">
-      <c r="A15" s="129" t="n"/>
-      <c r="B15" s="95" t="inlineStr">
+    <row r="15" ht="48" customFormat="1" customHeight="1" s="53" thickBot="1">
+      <c r="A15" s="178" t="n"/>
+      <c r="B15" s="237" t="inlineStr">
         <is>
           <t>Phase 2 - Chp</t>
         </is>
       </c>
-      <c r="C15" s="96" t="inlineStr">
+      <c r="C15" s="238" t="inlineStr">
         <is>
           <t>Phase 2: Chp</t>
         </is>
       </c>
-      <c r="D15" s="90" t="n"/>
-      <c r="E15" s="90" t="n"/>
-      <c r="F15" s="13" t="n"/>
-      <c r="G15" s="13">
+      <c r="D15" s="239" t="n"/>
+      <c r="E15" s="239" t="n"/>
+      <c r="F15" s="182" t="n"/>
+      <c r="G15" s="182">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v/>
       </c>
-      <c r="H15" s="56" t="n"/>
-      <c r="I15" s="55" t="n"/>
-      <c r="J15" s="55" t="n"/>
-      <c r="K15" s="55" t="n"/>
-      <c r="L15" s="55" t="n"/>
-      <c r="M15" s="55" t="n"/>
-      <c r="N15" s="55" t="n"/>
-      <c r="O15" s="55" t="n"/>
-      <c r="P15" s="55" t="n"/>
-      <c r="Q15" s="55" t="n"/>
-      <c r="R15" s="55" t="n"/>
-      <c r="S15" s="55" t="n"/>
-      <c r="T15" s="55" t="n"/>
-      <c r="U15" s="55" t="n"/>
-      <c r="V15" s="55" t="n"/>
-      <c r="W15" s="55" t="n"/>
-      <c r="X15" s="55" t="n"/>
-      <c r="Y15" s="55" t="n"/>
-      <c r="Z15" s="55" t="n"/>
-      <c r="AA15" s="55" t="n"/>
-      <c r="AB15" s="55" t="n"/>
-      <c r="AC15" s="55" t="n"/>
-      <c r="AD15" s="55" t="n"/>
-      <c r="AE15" s="55" t="n"/>
-      <c r="AF15" s="55" t="n"/>
-      <c r="AG15" s="55" t="n"/>
-      <c r="AH15" s="55" t="n"/>
-      <c r="AI15" s="55" t="n"/>
-      <c r="AJ15" s="55" t="n"/>
-      <c r="AK15" s="55" t="n"/>
-      <c r="AL15" s="55" t="n"/>
-      <c r="AM15" s="55" t="n"/>
-      <c r="AN15" s="55" t="n"/>
-      <c r="AO15" s="55" t="n"/>
-      <c r="AP15" s="55" t="n"/>
-      <c r="BG15" s="77" t="n"/>
+      <c r="H15" s="281" t="n"/>
+      <c r="I15" s="282" t="n"/>
+      <c r="J15" s="282" t="n"/>
+      <c r="K15" s="282" t="n"/>
+      <c r="L15" s="282" t="n"/>
+      <c r="M15" s="282" t="n"/>
+      <c r="N15" s="282" t="n"/>
+      <c r="O15" s="282" t="n"/>
+      <c r="P15" s="282" t="n"/>
+      <c r="Q15" s="282" t="n"/>
+      <c r="R15" s="282" t="n"/>
+      <c r="S15" s="282" t="n"/>
+      <c r="T15" s="282" t="n"/>
+      <c r="U15" s="282" t="n"/>
+      <c r="V15" s="282" t="n"/>
+      <c r="W15" s="282" t="n"/>
+      <c r="X15" s="282" t="n"/>
+      <c r="Y15" s="282" t="n"/>
+      <c r="Z15" s="282" t="n"/>
+      <c r="AA15" s="282" t="n"/>
+      <c r="AB15" s="282" t="n"/>
+      <c r="AC15" s="282" t="n"/>
+      <c r="AD15" s="282" t="n"/>
+      <c r="AE15" s="282" t="n"/>
+      <c r="AF15" s="282" t="n"/>
+      <c r="AG15" s="282" t="n"/>
+      <c r="AH15" s="282" t="n"/>
+      <c r="AI15" s="282" t="n"/>
+      <c r="AJ15" s="282" t="n"/>
+      <c r="AK15" s="282" t="n"/>
+      <c r="AL15" s="282" t="n"/>
+      <c r="AM15" s="282" t="n"/>
+      <c r="AN15" s="282" t="n"/>
+      <c r="AO15" s="282" t="n"/>
+      <c r="AP15" s="282" t="n"/>
+      <c r="AQ15" s="283" t="n"/>
+      <c r="AR15" s="283" t="n"/>
+      <c r="AS15" s="283" t="n"/>
+      <c r="AT15" s="283" t="n"/>
+      <c r="AU15" s="283" t="n"/>
+      <c r="AV15" s="283" t="n"/>
+      <c r="AW15" s="283" t="n"/>
+      <c r="AX15" s="283" t="n"/>
+      <c r="AY15" s="283" t="n"/>
+      <c r="AZ15" s="283" t="n"/>
+      <c r="BA15" s="283" t="n"/>
+      <c r="BB15" s="283" t="n"/>
+      <c r="BC15" s="283" t="n"/>
+      <c r="BD15" s="283" t="n"/>
+      <c r="BE15" s="284" t="n"/>
+      <c r="BF15" s="284" t="n"/>
+      <c r="BG15" s="156" t="n"/>
+      <c r="BH15" s="153" t="n"/>
+      <c r="BI15" s="153" t="n"/>
+      <c r="BJ15" s="153" t="n"/>
+      <c r="BK15" s="153" t="n"/>
+      <c r="BL15" s="153" t="n"/>
+      <c r="BM15" s="153" t="n"/>
+      <c r="BN15" s="153" t="n"/>
+      <c r="BO15" s="153" t="n"/>
+      <c r="BP15" s="153" t="n"/>
+      <c r="BQ15" s="153" t="n"/>
+      <c r="BR15" s="153" t="n"/>
+      <c r="BS15" s="153" t="n"/>
+      <c r="BT15" s="153" t="n"/>
+      <c r="BU15" s="153" t="n"/>
+      <c r="BV15" s="153" t="n"/>
+      <c r="BW15" s="153" t="n"/>
+      <c r="BX15" s="153" t="n"/>
+      <c r="BY15" s="153" t="n"/>
+      <c r="BZ15" s="153" t="n"/>
+      <c r="CA15" s="153" t="n"/>
     </row>
-    <row r="16" ht="20" customFormat="1" customHeight="1" s="53" thickBot="1">
-      <c r="A16" s="129" t="n"/>
-      <c r="B16" s="97" t="inlineStr">
+    <row r="16" ht="54" customFormat="1" customHeight="1" s="53" thickBot="1">
+      <c r="A16" s="178" t="n"/>
+      <c r="B16" s="268" t="inlineStr">
         <is>
           <t>Study 1: Evidence in Cyber Operations - A Thematic Review</t>
         </is>
       </c>
-      <c r="C16" s="98" t="n">
+      <c r="C16" s="269" t="n">
         <v>1</v>
       </c>
       <c r="D16" s="78" t="n">
-        <v>45383</v>
+        <v>45812</v>
       </c>
       <c r="E16" s="78" t="n">
-        <v>45930</v>
-      </c>
-      <c r="F16" s="13" t="n"/>
-      <c r="G16" s="13" t="n"/>
-      <c r="H16" s="64" t="n"/>
-      <c r="I16" s="132" t="n"/>
-      <c r="J16" s="132" t="n"/>
-      <c r="K16" s="132" t="n"/>
-      <c r="L16" s="132" t="n"/>
-      <c r="M16" s="132" t="n"/>
-      <c r="N16" s="132" t="n"/>
-      <c r="O16" s="132" t="n"/>
-      <c r="P16" s="132" t="n"/>
-      <c r="Q16" s="132" t="n"/>
-      <c r="R16" s="132" t="n"/>
-      <c r="S16" s="132" t="n"/>
-      <c r="T16" s="132" t="n"/>
-      <c r="U16" s="132" t="n"/>
-      <c r="V16" s="132" t="n"/>
-      <c r="W16" s="132" t="n"/>
-      <c r="X16" s="132" t="n"/>
-      <c r="Y16" s="132" t="n"/>
-      <c r="Z16" s="67" t="n"/>
-      <c r="AA16" s="140" t="inlineStr">
+        <v>45996</v>
+      </c>
+      <c r="F16" s="182" t="n"/>
+      <c r="G16" s="182" t="n"/>
+      <c r="H16" s="270" t="inlineStr">
         <is>
-          <t>Chp 1 -Introduction</t>
+          <t>Chp 1 - Introduction</t>
         </is>
       </c>
-      <c r="AI16" s="132" t="n"/>
-      <c r="AJ16" s="141" t="n"/>
-      <c r="AK16" s="132" t="n"/>
-      <c r="AL16" s="132" t="n"/>
-      <c r="AM16" s="132" t="n"/>
-      <c r="AN16" s="132" t="n"/>
-      <c r="AO16" s="132" t="n"/>
-      <c r="AP16" s="132" t="n"/>
-      <c r="AQ16" s="132" t="n"/>
-      <c r="AR16" s="132" t="n"/>
-      <c r="AS16" s="142" t="n"/>
-      <c r="AT16" s="132" t="n"/>
-      <c r="AU16" s="132" t="n"/>
-      <c r="AV16" s="132" t="n"/>
-      <c r="AW16" s="132" t="n"/>
-      <c r="AX16" s="132" t="n"/>
-      <c r="AY16" s="132" t="n"/>
-      <c r="AZ16" s="132" t="n"/>
-      <c r="BA16" s="132" t="n"/>
-      <c r="BB16" s="132" t="n"/>
-      <c r="BC16" s="132" t="n"/>
-      <c r="BD16" s="132" t="n"/>
-      <c r="BG16" s="77" t="n"/>
+      <c r="I16" s="290" t="n"/>
+      <c r="J16" s="290" t="n"/>
+      <c r="K16" s="290" t="n"/>
+      <c r="L16" s="290" t="n"/>
+      <c r="M16" s="290" t="n"/>
+      <c r="N16" s="290" t="n"/>
+      <c r="O16" s="290" t="n"/>
+      <c r="P16" s="290" t="n"/>
+      <c r="Q16" s="290" t="n"/>
+      <c r="R16" s="290" t="n"/>
+      <c r="S16" s="290" t="n"/>
+      <c r="T16" s="290" t="n"/>
+      <c r="U16" s="290" t="n"/>
+      <c r="V16" s="290" t="n"/>
+      <c r="W16" s="290" t="n"/>
+      <c r="X16" s="290" t="n"/>
+      <c r="Y16" s="290" t="n"/>
+      <c r="Z16" s="291" t="n"/>
+      <c r="AA16" s="273" t="n"/>
+      <c r="AB16" s="283" t="n"/>
+      <c r="AC16" s="283" t="n"/>
+      <c r="AD16" s="283" t="n"/>
+      <c r="AE16" s="283" t="n"/>
+      <c r="AF16" s="283" t="n"/>
+      <c r="AG16" s="283" t="n"/>
+      <c r="AH16" s="283" t="n"/>
+      <c r="AI16" s="290" t="n"/>
+      <c r="AJ16" s="274" t="n"/>
+      <c r="AK16" s="290" t="n"/>
+      <c r="AL16" s="290" t="n"/>
+      <c r="AM16" s="290" t="n"/>
+      <c r="AN16" s="290" t="n"/>
+      <c r="AO16" s="275" t="n"/>
+      <c r="AP16" s="290" t="n"/>
+      <c r="AQ16" s="290" t="n"/>
+      <c r="AR16" s="290" t="n"/>
+      <c r="AS16" s="276" t="n"/>
+      <c r="AT16" s="290" t="n"/>
+      <c r="AU16" s="290" t="n"/>
+      <c r="AV16" s="290" t="n"/>
+      <c r="AW16" s="290" t="n"/>
+      <c r="AX16" s="290" t="n"/>
+      <c r="AY16" s="290" t="n"/>
+      <c r="AZ16" s="290" t="n"/>
+      <c r="BA16" s="290" t="n"/>
+      <c r="BB16" s="290" t="n"/>
+      <c r="BC16" s="290" t="n"/>
+      <c r="BD16" s="290" t="n"/>
+      <c r="BE16" s="284" t="n"/>
+      <c r="BF16" s="284" t="n"/>
+      <c r="BG16" s="156" t="n"/>
+      <c r="BH16" s="153" t="n"/>
+      <c r="BI16" s="153" t="n"/>
+      <c r="BJ16" s="153" t="n"/>
+      <c r="BK16" s="153" t="n"/>
+      <c r="BL16" s="153" t="n"/>
+      <c r="BM16" s="153" t="n"/>
+      <c r="BN16" s="153" t="n"/>
+      <c r="BO16" s="153" t="n"/>
+      <c r="BP16" s="153" t="n"/>
+      <c r="BQ16" s="153" t="n"/>
+      <c r="BR16" s="153" t="n"/>
+      <c r="BS16" s="153" t="n"/>
+      <c r="BT16" s="153" t="n"/>
+      <c r="BU16" s="153" t="n"/>
+      <c r="BV16" s="153" t="n"/>
+      <c r="BW16" s="153" t="n"/>
+      <c r="BX16" s="153" t="n"/>
+      <c r="BY16" s="153" t="n"/>
+      <c r="BZ16" s="153" t="n"/>
+      <c r="CA16" s="153" t="n"/>
     </row>
-    <row r="17" ht="20" customFormat="1" customHeight="1" s="53" thickBot="1">
-      <c r="A17" s="129" t="n"/>
-      <c r="B17" s="97" t="inlineStr">
+    <row r="17" ht="54" customFormat="1" customHeight="1" s="53" thickBot="1">
+      <c r="A17" s="178" t="n"/>
+      <c r="B17" s="268" t="inlineStr">
         <is>
           <t>Study 1: Evidence in Cyber Operations - Manuscript Revision</t>
         </is>
       </c>
-      <c r="C17" s="98" t="n">
-        <v>1</v>
+      <c r="C17" s="269" t="n">
+        <v>0.8</v>
       </c>
       <c r="D17" s="78" t="n">
-        <v>45383</v>
+        <v>45812</v>
       </c>
       <c r="E17" s="78" t="n">
-        <v>46021</v>
-      </c>
-      <c r="F17" s="13" t="n"/>
-      <c r="G17" s="13" t="n"/>
-      <c r="H17" s="64" t="n"/>
-      <c r="I17" s="132" t="n"/>
-      <c r="J17" s="132" t="n"/>
-      <c r="K17" s="132" t="n"/>
-      <c r="L17" s="132" t="n"/>
-      <c r="M17" s="132" t="n"/>
-      <c r="N17" s="132" t="n"/>
-      <c r="O17" s="132" t="n"/>
-      <c r="P17" s="132" t="n"/>
-      <c r="Q17" s="132" t="n"/>
-      <c r="R17" s="132" t="n"/>
-      <c r="S17" s="132" t="n"/>
-      <c r="T17" s="132" t="n"/>
-      <c r="U17" s="132" t="n"/>
-      <c r="V17" s="132" t="n"/>
-      <c r="W17" s="132" t="n"/>
-      <c r="X17" s="132" t="n"/>
-      <c r="Y17" s="132" t="n"/>
-      <c r="Z17" s="67" t="n"/>
-      <c r="AA17" s="140" t="inlineStr">
+        <v>46113</v>
+      </c>
+      <c r="F17" s="182" t="n"/>
+      <c r="G17" s="182" t="n"/>
+      <c r="H17" s="270" t="inlineStr">
         <is>
-          <t>Chp 2 - Systematic Review</t>
+          <t>Chp 2 - Methods and Concepts</t>
         </is>
       </c>
-      <c r="AI17" s="132" t="n"/>
-      <c r="AJ17" s="132" t="n"/>
-      <c r="AK17" s="141" t="n"/>
-      <c r="AL17" s="132" t="n"/>
-      <c r="AM17" s="132" t="n"/>
-      <c r="AN17" s="132" t="n"/>
-      <c r="AO17" s="132" t="n"/>
-      <c r="AP17" s="132" t="n"/>
-      <c r="AQ17" s="132" t="n"/>
-      <c r="AR17" s="132" t="n"/>
-      <c r="AS17" s="132" t="n"/>
-      <c r="AT17" s="132" t="n"/>
-      <c r="AU17" s="132" t="n"/>
-      <c r="AV17" s="142" t="n"/>
-      <c r="AW17" s="132" t="n"/>
-      <c r="AX17" s="132" t="n"/>
-      <c r="AY17" s="132" t="n"/>
-      <c r="AZ17" s="132" t="n"/>
-      <c r="BA17" s="132" t="n"/>
-      <c r="BB17" s="132" t="n"/>
-      <c r="BC17" s="132" t="n"/>
-      <c r="BD17" s="132" t="n"/>
-      <c r="BG17" s="77" t="n"/>
+      <c r="I17" s="290" t="n"/>
+      <c r="J17" s="290" t="n"/>
+      <c r="K17" s="290" t="n"/>
+      <c r="L17" s="290" t="n"/>
+      <c r="M17" s="290" t="n"/>
+      <c r="N17" s="290" t="n"/>
+      <c r="O17" s="290" t="n"/>
+      <c r="P17" s="290" t="n"/>
+      <c r="Q17" s="290" t="n"/>
+      <c r="R17" s="290" t="n"/>
+      <c r="S17" s="290" t="n"/>
+      <c r="T17" s="290" t="n"/>
+      <c r="U17" s="290" t="n"/>
+      <c r="V17" s="290" t="n"/>
+      <c r="W17" s="290" t="n"/>
+      <c r="X17" s="290" t="n"/>
+      <c r="Y17" s="290" t="n"/>
+      <c r="Z17" s="291" t="n"/>
+      <c r="AA17" s="273" t="n"/>
+      <c r="AB17" s="283" t="n"/>
+      <c r="AC17" s="283" t="n"/>
+      <c r="AD17" s="283" t="n"/>
+      <c r="AE17" s="283" t="n"/>
+      <c r="AF17" s="283" t="n"/>
+      <c r="AG17" s="283" t="n"/>
+      <c r="AH17" s="283" t="n"/>
+      <c r="AI17" s="290" t="n"/>
+      <c r="AJ17" s="290" t="n"/>
+      <c r="AK17" s="274" t="n"/>
+      <c r="AL17" s="290" t="n"/>
+      <c r="AM17" s="290" t="n"/>
+      <c r="AN17" s="290" t="n"/>
+      <c r="AO17" s="275" t="n"/>
+      <c r="AP17" s="290" t="n"/>
+      <c r="AQ17" s="290" t="n"/>
+      <c r="AR17" s="290" t="n"/>
+      <c r="AS17" s="290" t="n"/>
+      <c r="AT17" s="290" t="n"/>
+      <c r="AU17" s="290" t="n"/>
+      <c r="AV17" s="276" t="n"/>
+      <c r="AW17" s="290" t="n"/>
+      <c r="AX17" s="290" t="n"/>
+      <c r="AY17" s="290" t="n"/>
+      <c r="AZ17" s="290" t="n"/>
+      <c r="BA17" s="290" t="n"/>
+      <c r="BB17" s="290" t="n"/>
+      <c r="BC17" s="290" t="n"/>
+      <c r="BD17" s="290" t="n"/>
+      <c r="BE17" s="284" t="n"/>
+      <c r="BF17" s="284" t="n"/>
+      <c r="BG17" s="156" t="n"/>
+      <c r="BH17" s="153" t="n"/>
+      <c r="BI17" s="153" t="n"/>
+      <c r="BJ17" s="153" t="n"/>
+      <c r="BK17" s="153" t="n"/>
+      <c r="BL17" s="153" t="n"/>
+      <c r="BM17" s="153" t="n"/>
+      <c r="BN17" s="153" t="n"/>
+      <c r="BO17" s="153" t="n"/>
+      <c r="BP17" s="153" t="n"/>
+      <c r="BQ17" s="153" t="n"/>
+      <c r="BR17" s="153" t="n"/>
+      <c r="BS17" s="153" t="n"/>
+      <c r="BT17" s="153" t="n"/>
+      <c r="BU17" s="153" t="n"/>
+      <c r="BV17" s="153" t="n"/>
+      <c r="BW17" s="153" t="n"/>
+      <c r="BX17" s="153" t="n"/>
+      <c r="BY17" s="153" t="n"/>
+      <c r="BZ17" s="153" t="n"/>
+      <c r="CA17" s="153" t="n"/>
     </row>
-    <row r="18" ht="20" customFormat="1" customHeight="1" s="53" thickBot="1">
-      <c r="A18" s="130" t="n"/>
-      <c r="B18" s="97" t="inlineStr">
+    <row r="18" ht="54" customFormat="1" customHeight="1" s="53" thickBot="1">
+      <c r="A18" s="197" t="n"/>
+      <c r="B18" s="268" t="inlineStr">
         <is>
           <t>Study 2: Applications of Zero-Knowledge-Proofs to Social Science</t>
         </is>
       </c>
-      <c r="C18" s="98" t="n">
-        <v>0.9</v>
+      <c r="C18" s="269" t="n">
+        <v>0.8</v>
       </c>
       <c r="D18" s="78" t="n">
-        <v>45931</v>
+        <v>45779</v>
       </c>
       <c r="E18" s="78" t="n">
-        <v>46081</v>
-      </c>
-      <c r="F18" s="13" t="n"/>
-      <c r="G18" s="63">
+        <v>46144</v>
+      </c>
+      <c r="F18" s="182" t="n"/>
+      <c r="G18" s="211">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v/>
       </c>
-      <c r="H18" s="64" t="n"/>
-      <c r="I18" s="64" t="n"/>
-      <c r="J18" s="64" t="n"/>
-      <c r="K18" s="64" t="n"/>
-      <c r="L18" s="64" t="n"/>
-      <c r="M18" s="64" t="n"/>
-      <c r="N18" s="64" t="n"/>
-      <c r="O18" s="64" t="n"/>
-      <c r="P18" s="64" t="n"/>
-      <c r="Q18" s="64" t="n"/>
-      <c r="R18" s="64" t="n"/>
-      <c r="S18" s="64" t="n"/>
-      <c r="T18" s="66" t="n"/>
-      <c r="U18" s="66" t="n"/>
-      <c r="V18" s="64" t="n"/>
-      <c r="W18" s="64" t="n"/>
-      <c r="X18" s="64" t="n"/>
-      <c r="Y18" s="64" t="n"/>
-      <c r="Z18" s="64" t="n"/>
-      <c r="AA18" s="64" t="n"/>
-      <c r="AB18" s="64" t="n"/>
-      <c r="AC18" s="64" t="n"/>
-      <c r="AD18" s="64" t="n"/>
-      <c r="AE18" s="64" t="n"/>
-      <c r="AF18" s="64" t="n"/>
-      <c r="AG18" s="64" t="n"/>
-      <c r="AH18" s="64" t="n"/>
-      <c r="AI18" s="64" t="n"/>
-      <c r="AJ18" s="64" t="n"/>
-      <c r="AK18" s="64" t="n"/>
-      <c r="AL18" s="64" t="n"/>
-      <c r="AM18" s="64" t="n"/>
-      <c r="AN18" s="64" t="n"/>
-      <c r="AO18" s="64" t="n"/>
-      <c r="AP18" s="64" t="n"/>
-      <c r="AQ18" s="64" t="n"/>
-      <c r="AR18" s="64" t="n"/>
-      <c r="AS18" s="140" t="inlineStr">
+      <c r="H18" s="270" t="inlineStr">
         <is>
-          <t>Chp3: Methods and Concepts</t>
+          <t>Chp 3 - A Systematic Evolution of Cyber-Attribution Scholarship (2001-2025)</t>
         </is>
       </c>
-      <c r="BA18" s="64" t="n"/>
-      <c r="BB18" s="64" t="n"/>
-      <c r="BC18" s="64" t="n"/>
-      <c r="BD18" s="64" t="n"/>
-      <c r="BG18" s="77" t="n"/>
+      <c r="I18" s="282" t="n"/>
+      <c r="J18" s="282" t="n"/>
+      <c r="K18" s="282" t="n"/>
+      <c r="L18" s="282" t="n"/>
+      <c r="M18" s="282" t="n"/>
+      <c r="N18" s="282" t="n"/>
+      <c r="O18" s="282" t="n"/>
+      <c r="P18" s="282" t="n"/>
+      <c r="Q18" s="282" t="n"/>
+      <c r="R18" s="282" t="n"/>
+      <c r="S18" s="282" t="n"/>
+      <c r="T18" s="292" t="n"/>
+      <c r="U18" s="292" t="n"/>
+      <c r="V18" s="282" t="n"/>
+      <c r="W18" s="282" t="n"/>
+      <c r="X18" s="282" t="n"/>
+      <c r="Y18" s="282" t="n"/>
+      <c r="Z18" s="282" t="n"/>
+      <c r="AA18" s="282" t="n"/>
+      <c r="AB18" s="282" t="n"/>
+      <c r="AC18" s="282" t="n"/>
+      <c r="AD18" s="282" t="n"/>
+      <c r="AE18" s="282" t="n"/>
+      <c r="AF18" s="282" t="n"/>
+      <c r="AG18" s="282" t="n"/>
+      <c r="AH18" s="282" t="n"/>
+      <c r="AI18" s="282" t="n"/>
+      <c r="AJ18" s="282" t="n"/>
+      <c r="AK18" s="282" t="n"/>
+      <c r="AL18" s="282" t="n"/>
+      <c r="AM18" s="282" t="n"/>
+      <c r="AN18" s="275" t="n"/>
+      <c r="AO18" s="282" t="n"/>
+      <c r="AP18" s="282" t="n"/>
+      <c r="AQ18" s="282" t="n"/>
+      <c r="AR18" s="282" t="n"/>
+      <c r="AS18" s="273" t="n"/>
+      <c r="AT18" s="283" t="n"/>
+      <c r="AU18" s="283" t="n"/>
+      <c r="AV18" s="283" t="n"/>
+      <c r="AW18" s="283" t="n"/>
+      <c r="AX18" s="283" t="n"/>
+      <c r="AY18" s="283" t="n"/>
+      <c r="AZ18" s="283" t="n"/>
+      <c r="BA18" s="282" t="n"/>
+      <c r="BB18" s="282" t="n"/>
+      <c r="BC18" s="282" t="n"/>
+      <c r="BD18" s="282" t="n"/>
+      <c r="BE18" s="284" t="n"/>
+      <c r="BF18" s="284" t="n"/>
+      <c r="BG18" s="156" t="n"/>
+      <c r="BH18" s="153" t="n"/>
+      <c r="BI18" s="153" t="n"/>
+      <c r="BJ18" s="153" t="n"/>
+      <c r="BK18" s="153" t="n"/>
+      <c r="BL18" s="153" t="n"/>
+      <c r="BM18" s="153" t="n"/>
+      <c r="BN18" s="153" t="n"/>
+      <c r="BO18" s="153" t="n"/>
+      <c r="BP18" s="153" t="n"/>
+      <c r="BQ18" s="153" t="n"/>
+      <c r="BR18" s="153" t="n"/>
+      <c r="BS18" s="153" t="n"/>
+      <c r="BT18" s="153" t="n"/>
+      <c r="BU18" s="153" t="n"/>
+      <c r="BV18" s="153" t="n"/>
+      <c r="BW18" s="153" t="n"/>
+      <c r="BX18" s="153" t="n"/>
+      <c r="BY18" s="153" t="n"/>
+      <c r="BZ18" s="153" t="n"/>
+      <c r="CA18" s="153" t="n"/>
     </row>
-    <row r="19" ht="20" customFormat="1" customHeight="1" s="53" thickBot="1">
-      <c r="A19" s="130" t="n"/>
-      <c r="B19" s="97" t="inlineStr">
+    <row r="19" ht="54" customFormat="1" customHeight="1" s="53" thickBot="1">
+      <c r="A19" s="197" t="n"/>
+      <c r="B19" s="268" t="inlineStr">
         <is>
           <t>Study 3: Cyber Due Diligence as a Standard for Attribution</t>
         </is>
       </c>
-      <c r="C19" s="98" t="n">
+      <c r="C19" s="269" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="78" t="n">
@@ -3560,366 +4456,462 @@
       <c r="E19" s="78" t="n">
         <v>45960</v>
       </c>
-      <c r="F19" s="13" t="n"/>
-      <c r="G19" s="3">
+      <c r="F19" s="182" t="n"/>
+      <c r="G19" s="183">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v/>
       </c>
-      <c r="H19" s="64" t="n"/>
-      <c r="I19" s="64" t="n"/>
-      <c r="J19" s="64" t="n"/>
-      <c r="K19" s="64" t="n"/>
-      <c r="L19" s="140" t="inlineStr">
+      <c r="H19" s="270" t="inlineStr">
         <is>
-          <t>Chp4: ZKPs and IR (1 article)</t>
+          <t>Chp 4 - Zero Knowledge Proofs in the Attribution of International Cyber Incidents: The value of opacity</t>
         </is>
       </c>
-      <c r="T19" s="64" t="n"/>
-      <c r="U19" s="64" t="n"/>
-      <c r="V19" s="64" t="n"/>
-      <c r="W19" s="64" t="n"/>
-      <c r="X19" s="64" t="n"/>
-      <c r="Y19" s="64" t="n"/>
-      <c r="Z19" s="64" t="n"/>
-      <c r="AA19" s="64" t="n"/>
-      <c r="AB19" s="64" t="n"/>
-      <c r="AC19" s="141" t="n"/>
-      <c r="AD19" s="64" t="n"/>
-      <c r="AE19" s="64" t="n"/>
-      <c r="AF19" s="64" t="n"/>
-      <c r="AG19" s="64" t="n"/>
-      <c r="AH19" s="64" t="n"/>
-      <c r="AI19" s="64" t="n"/>
-      <c r="AJ19" s="64" t="n"/>
-      <c r="AK19" s="64" t="n"/>
-      <c r="AL19" s="64" t="n"/>
-      <c r="AM19" s="64" t="n"/>
-      <c r="AN19" s="64" t="n"/>
-      <c r="AO19" s="64" t="n"/>
-      <c r="AP19" s="64" t="n"/>
-      <c r="AQ19" s="64" t="n"/>
-      <c r="AR19" s="64" t="n"/>
-      <c r="AS19" s="64" t="n"/>
-      <c r="AT19" s="142" t="n"/>
-      <c r="AU19" s="64" t="n"/>
-      <c r="AV19" s="64" t="n"/>
-      <c r="AW19" s="64" t="n"/>
-      <c r="AX19" s="64" t="n"/>
-      <c r="AY19" s="64" t="n"/>
-      <c r="AZ19" s="64" t="n"/>
-      <c r="BA19" s="64" t="n"/>
-      <c r="BB19" s="64" t="n"/>
-      <c r="BC19" s="64" t="n"/>
-      <c r="BD19" s="64" t="n"/>
-      <c r="BG19" s="77" t="n"/>
+      <c r="I19" s="282" t="n"/>
+      <c r="J19" s="282" t="n"/>
+      <c r="K19" s="282" t="n"/>
+      <c r="L19" s="275" t="n"/>
+      <c r="M19" s="283" t="n"/>
+      <c r="N19" s="283" t="n"/>
+      <c r="O19" s="283" t="n"/>
+      <c r="P19" s="283" t="n"/>
+      <c r="Q19" s="283" t="n"/>
+      <c r="R19" s="283" t="n"/>
+      <c r="S19" s="283" t="n"/>
+      <c r="T19" s="282" t="n"/>
+      <c r="U19" s="282" t="n"/>
+      <c r="V19" s="282" t="n"/>
+      <c r="W19" s="282" t="n"/>
+      <c r="X19" s="282" t="n"/>
+      <c r="Y19" s="282" t="n"/>
+      <c r="Z19" s="282" t="n"/>
+      <c r="AA19" s="282" t="n"/>
+      <c r="AB19" s="282" t="n"/>
+      <c r="AC19" s="274" t="n"/>
+      <c r="AD19" s="282" t="n"/>
+      <c r="AE19" s="282" t="n"/>
+      <c r="AF19" s="282" t="n"/>
+      <c r="AG19" s="282" t="n"/>
+      <c r="AH19" s="282" t="n"/>
+      <c r="AI19" s="282" t="n"/>
+      <c r="AJ19" s="282" t="n"/>
+      <c r="AK19" s="282" t="n"/>
+      <c r="AL19" s="282" t="n"/>
+      <c r="AM19" s="282" t="n"/>
+      <c r="AN19" s="282" t="n"/>
+      <c r="AO19" s="282" t="n"/>
+      <c r="AP19" s="282" t="n"/>
+      <c r="AQ19" s="282" t="n"/>
+      <c r="AR19" s="282" t="n"/>
+      <c r="AS19" s="282" t="n"/>
+      <c r="AT19" s="276" t="n"/>
+      <c r="AU19" s="282" t="n"/>
+      <c r="AV19" s="282" t="n"/>
+      <c r="AW19" s="282" t="n"/>
+      <c r="AX19" s="282" t="n"/>
+      <c r="AY19" s="282" t="n"/>
+      <c r="AZ19" s="282" t="n"/>
+      <c r="BA19" s="282" t="n"/>
+      <c r="BB19" s="282" t="n"/>
+      <c r="BC19" s="282" t="n"/>
+      <c r="BD19" s="282" t="n"/>
+      <c r="BE19" s="284" t="n"/>
+      <c r="BF19" s="284" t="n"/>
+      <c r="BG19" s="156" t="n"/>
+      <c r="BH19" s="153" t="n"/>
+      <c r="BI19" s="153" t="n"/>
+      <c r="BJ19" s="153" t="n"/>
+      <c r="BK19" s="153" t="n"/>
+      <c r="BL19" s="153" t="n"/>
+      <c r="BM19" s="153" t="n"/>
+      <c r="BN19" s="153" t="n"/>
+      <c r="BO19" s="153" t="n"/>
+      <c r="BP19" s="153" t="n"/>
+      <c r="BQ19" s="153" t="n"/>
+      <c r="BR19" s="153" t="n"/>
+      <c r="BS19" s="153" t="n"/>
+      <c r="BT19" s="153" t="n"/>
+      <c r="BU19" s="153" t="n"/>
+      <c r="BV19" s="153" t="n"/>
+      <c r="BW19" s="153" t="n"/>
+      <c r="BX19" s="153" t="n"/>
+      <c r="BY19" s="153" t="n"/>
+      <c r="BZ19" s="153" t="n"/>
+      <c r="CA19" s="153" t="n"/>
     </row>
-    <row r="20" ht="20" customFormat="1" customHeight="1" s="53" thickBot="1">
-      <c r="A20" s="130" t="n"/>
-      <c r="B20" s="97" t="inlineStr">
+    <row r="20" ht="54" customFormat="1" customHeight="1" s="53" thickBot="1">
+      <c r="A20" s="197" t="n"/>
+      <c r="B20" s="268" t="inlineStr">
         <is>
           <t>Article 1: Attribution of Cyber Incidents in International Politics</t>
         </is>
       </c>
-      <c r="C20" s="98" t="n">
+      <c r="C20" s="269" t="n">
         <v>1</v>
       </c>
       <c r="D20" s="78" t="n">
-        <v>45369</v>
+        <v>45908</v>
       </c>
       <c r="E20" s="78" t="n">
-        <v>45979</v>
-      </c>
-      <c r="F20" s="13" t="n"/>
-      <c r="G20" s="3">
+        <v>46106</v>
+      </c>
+      <c r="F20" s="182" t="n"/>
+      <c r="G20" s="183">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v/>
       </c>
-      <c r="H20" s="64" t="n"/>
-      <c r="I20" s="64" t="n"/>
-      <c r="J20" s="64" t="n"/>
-      <c r="K20" s="64" t="n"/>
-      <c r="L20" s="64" t="n"/>
-      <c r="M20" s="64" t="n"/>
-      <c r="N20" s="64" t="n"/>
-      <c r="O20" s="64" t="n"/>
-      <c r="P20" s="64" t="n"/>
-      <c r="Q20" s="64" t="n"/>
-      <c r="R20" s="64" t="n"/>
-      <c r="S20" s="64" t="n"/>
-      <c r="T20" s="64" t="n"/>
-      <c r="U20" s="64" t="n"/>
-      <c r="V20" s="64" t="n"/>
-      <c r="W20" s="132" t="n"/>
-      <c r="Z20" s="143" t="inlineStr">
+      <c r="H20" s="270" t="inlineStr">
         <is>
-          <t>Chp5: Attribution Framework (two articles)</t>
+          <t>Chp 5 - Reframing Evidence in Cyber Attribution: The 3C Framework</t>
         </is>
       </c>
-      <c r="AH20" s="64" t="n"/>
-      <c r="AI20" s="64" t="n"/>
-      <c r="AJ20" s="141" t="n"/>
-      <c r="AK20" s="64" t="n"/>
-      <c r="AL20" s="64" t="n"/>
-      <c r="AM20" s="64" t="n"/>
-      <c r="AN20" s="64" t="n"/>
-      <c r="AO20" s="64" t="n"/>
-      <c r="AP20" s="64" t="n"/>
-      <c r="AQ20" s="64" t="n"/>
-      <c r="AR20" s="64" t="n"/>
-      <c r="AS20" s="64" t="n"/>
-      <c r="AT20" s="142" t="n"/>
-      <c r="AU20" s="64" t="n"/>
-      <c r="AV20" s="64" t="n"/>
-      <c r="AW20" s="64" t="n"/>
-      <c r="AX20" s="64" t="n"/>
-      <c r="AY20" s="64" t="n"/>
-      <c r="AZ20" s="64" t="n"/>
-      <c r="BA20" s="64" t="n"/>
-      <c r="BB20" s="64" t="n"/>
-      <c r="BC20" s="64" t="n"/>
-      <c r="BD20" s="64" t="n"/>
-      <c r="BE20" s="60" t="n"/>
-      <c r="BF20" s="33" t="n"/>
-      <c r="BG20" s="80" t="n"/>
-      <c r="BH20" s="60" t="n"/>
-      <c r="BI20" s="33" t="n"/>
-      <c r="BJ20" s="33" t="n"/>
-      <c r="BK20" s="33" t="n"/>
-      <c r="BL20" s="33" t="n"/>
-      <c r="BM20" s="33" t="n"/>
-      <c r="BN20" s="33" t="n"/>
-      <c r="BO20" s="33" t="n"/>
+      <c r="I20" s="282" t="n"/>
+      <c r="J20" s="282" t="n"/>
+      <c r="K20" s="282" t="n"/>
+      <c r="L20" s="282" t="n"/>
+      <c r="M20" s="282" t="n"/>
+      <c r="N20" s="282" t="n"/>
+      <c r="O20" s="282" t="n"/>
+      <c r="P20" s="282" t="n"/>
+      <c r="Q20" s="282" t="n"/>
+      <c r="R20" s="282" t="n"/>
+      <c r="S20" s="282" t="n"/>
+      <c r="T20" s="282" t="n"/>
+      <c r="U20" s="282" t="n"/>
+      <c r="V20" s="282" t="n"/>
+      <c r="W20" s="290" t="n"/>
+      <c r="X20" s="283" t="n"/>
+      <c r="Y20" s="283" t="n"/>
+      <c r="Z20" s="273" t="n"/>
+      <c r="AA20" s="283" t="n"/>
+      <c r="AB20" s="283" t="n"/>
+      <c r="AC20" s="283" t="n"/>
+      <c r="AD20" s="283" t="n"/>
+      <c r="AE20" s="283" t="n"/>
+      <c r="AF20" s="283" t="n"/>
+      <c r="AG20" s="283" t="n"/>
+      <c r="AH20" s="282" t="n"/>
+      <c r="AI20" s="282" t="n"/>
+      <c r="AJ20" s="274" t="n"/>
+      <c r="AK20" s="282" t="n"/>
+      <c r="AL20" s="282" t="n"/>
+      <c r="AM20" s="282" t="n"/>
+      <c r="AN20" s="282" t="n"/>
+      <c r="AO20" s="282" t="n"/>
+      <c r="AP20" s="282" t="n"/>
+      <c r="AQ20" s="282" t="n"/>
+      <c r="AR20" s="275" t="n"/>
+      <c r="AS20" s="282" t="n"/>
+      <c r="AT20" s="276" t="n"/>
+      <c r="AU20" s="282" t="n"/>
+      <c r="AV20" s="282" t="n"/>
+      <c r="AW20" s="282" t="n"/>
+      <c r="AX20" s="282" t="n"/>
+      <c r="AY20" s="282" t="n"/>
+      <c r="AZ20" s="282" t="n"/>
+      <c r="BA20" s="282" t="n"/>
+      <c r="BB20" s="282" t="n"/>
+      <c r="BC20" s="282" t="n"/>
+      <c r="BD20" s="282" t="n"/>
+      <c r="BE20" s="288" t="n"/>
+      <c r="BF20" s="289" t="n"/>
+      <c r="BG20" s="156" t="n"/>
+      <c r="BH20" s="156" t="n"/>
+      <c r="BI20" s="156" t="n"/>
+      <c r="BJ20" s="156" t="n"/>
+      <c r="BK20" s="156" t="n"/>
+      <c r="BL20" s="156" t="n"/>
+      <c r="BM20" s="156" t="n"/>
+      <c r="BN20" s="156" t="n"/>
+      <c r="BO20" s="156" t="n"/>
+      <c r="BP20" s="153" t="n"/>
+      <c r="BQ20" s="153" t="n"/>
+      <c r="BR20" s="153" t="n"/>
+      <c r="BS20" s="153" t="n"/>
+      <c r="BT20" s="153" t="n"/>
+      <c r="BU20" s="153" t="n"/>
+      <c r="BV20" s="153" t="n"/>
+      <c r="BW20" s="153" t="n"/>
+      <c r="BX20" s="153" t="n"/>
+      <c r="BY20" s="153" t="n"/>
+      <c r="BZ20" s="153" t="n"/>
+      <c r="CA20" s="153" t="n"/>
     </row>
-    <row r="21" ht="20" customFormat="1" customHeight="1" s="53" thickBot="1">
-      <c r="A21" s="130" t="n"/>
-      <c r="B21" s="97" t="inlineStr">
+    <row r="21" ht="54" customFormat="1" customHeight="1" s="53" thickBot="1">
+      <c r="A21" s="197" t="n"/>
+      <c r="B21" s="268" t="inlineStr">
         <is>
           <t>Zero-knowledge attribution and international law - meeting the standard of proof in cyberspace</t>
         </is>
       </c>
-      <c r="C21" s="98" t="n">
+      <c r="C21" s="269" t="n">
         <v>1</v>
       </c>
       <c r="D21" s="78" t="n">
-        <v>45612</v>
+        <v>45602</v>
       </c>
       <c r="E21" s="78" t="n">
-        <v>45716</v>
-      </c>
-      <c r="F21" s="13" t="n"/>
-      <c r="G21" s="3">
+        <v>45935</v>
+      </c>
+      <c r="F21" s="182" t="n"/>
+      <c r="G21" s="183">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v/>
       </c>
-      <c r="H21" s="64" t="n"/>
-      <c r="I21" s="64" t="n"/>
-      <c r="J21" s="64" t="n"/>
-      <c r="K21" s="64" t="n"/>
-      <c r="L21" s="64" t="n"/>
-      <c r="M21" s="64" t="n"/>
-      <c r="N21" s="64" t="n"/>
-      <c r="O21" s="64" t="n"/>
-      <c r="P21" s="64" t="n"/>
-      <c r="Q21" s="64" t="n"/>
-      <c r="R21" s="64" t="n"/>
-      <c r="S21" s="64" t="n"/>
-      <c r="T21" s="64" t="n"/>
-      <c r="U21" s="64" t="n"/>
-      <c r="V21" s="64" t="n"/>
-      <c r="W21" s="64" t="n"/>
-      <c r="X21" s="64" t="n"/>
-      <c r="Y21" s="64" t="n"/>
-      <c r="Z21" s="64" t="n"/>
-      <c r="AA21" s="64" t="n"/>
-      <c r="AB21" s="64" t="n"/>
-      <c r="AC21" s="64" t="n"/>
-      <c r="AD21" s="64" t="n"/>
-      <c r="AE21" s="64" t="n"/>
-      <c r="AF21" s="64" t="n"/>
-      <c r="AG21" s="64" t="n"/>
-      <c r="AH21" s="140" t="inlineStr">
+      <c r="H21" s="270" t="inlineStr">
         <is>
-          <t>Chp6: Cyber attribution case before the ICJ (1 article)</t>
+          <t>Chp 6 - Secrecy in International Adjudication A Zero-Knowledge Cyber Attribution Case before the ICJ</t>
         </is>
       </c>
-      <c r="AP21" s="64" t="n"/>
-      <c r="AQ21" s="64" t="n"/>
-      <c r="AR21" s="64" t="n"/>
-      <c r="AS21" s="64" t="n"/>
-      <c r="AT21" s="64" t="n"/>
-      <c r="AU21" s="64" t="n"/>
-      <c r="AV21" s="64" t="n"/>
-      <c r="AW21" s="64" t="n"/>
-      <c r="AX21" s="64" t="n"/>
-      <c r="AY21" s="64" t="n"/>
-      <c r="AZ21" s="64" t="n"/>
-      <c r="BA21" s="64" t="n"/>
-      <c r="BB21" s="64" t="n"/>
-      <c r="BC21" s="64" t="n"/>
-      <c r="BD21" s="64" t="n"/>
-      <c r="BE21" s="60" t="n"/>
-      <c r="BF21" s="33" t="n"/>
-      <c r="BG21" s="80" t="n"/>
-      <c r="BH21" s="60" t="n"/>
-      <c r="BI21" s="33" t="n"/>
-      <c r="BJ21" s="33" t="n"/>
-      <c r="BK21" s="33" t="n"/>
-      <c r="BL21" s="33" t="n"/>
-      <c r="BM21" s="33" t="n"/>
-      <c r="BN21" s="33" t="n"/>
-      <c r="BO21" s="33" t="n"/>
+      <c r="I21" s="282" t="n"/>
+      <c r="J21" s="282" t="n"/>
+      <c r="K21" s="282" t="n"/>
+      <c r="L21" s="282" t="n"/>
+      <c r="M21" s="282" t="n"/>
+      <c r="N21" s="282" t="n"/>
+      <c r="O21" s="282" t="n"/>
+      <c r="P21" s="282" t="n"/>
+      <c r="Q21" s="282" t="n"/>
+      <c r="R21" s="282" t="n"/>
+      <c r="S21" s="282" t="n"/>
+      <c r="T21" s="282" t="n"/>
+      <c r="U21" s="282" t="n"/>
+      <c r="V21" s="282" t="n"/>
+      <c r="W21" s="282" t="n"/>
+      <c r="X21" s="282" t="n"/>
+      <c r="Y21" s="282" t="n"/>
+      <c r="Z21" s="282" t="n"/>
+      <c r="AA21" s="282" t="n"/>
+      <c r="AB21" s="282" t="n"/>
+      <c r="AC21" s="282" t="n"/>
+      <c r="AD21" s="282" t="n"/>
+      <c r="AE21" s="282" t="n"/>
+      <c r="AF21" s="282" t="n"/>
+      <c r="AG21" s="282" t="n"/>
+      <c r="AH21" s="275" t="n"/>
+      <c r="AI21" s="283" t="n"/>
+      <c r="AJ21" s="283" t="n"/>
+      <c r="AK21" s="283" t="n"/>
+      <c r="AL21" s="283" t="n"/>
+      <c r="AM21" s="283" t="n"/>
+      <c r="AN21" s="283" t="n"/>
+      <c r="AO21" s="283" t="n"/>
+      <c r="AP21" s="282" t="n"/>
+      <c r="AQ21" s="282" t="n"/>
+      <c r="AR21" s="282" t="n"/>
+      <c r="AS21" s="282" t="n"/>
+      <c r="AT21" s="282" t="n"/>
+      <c r="AU21" s="282" t="n"/>
+      <c r="AV21" s="282" t="n"/>
+      <c r="AW21" s="282" t="n"/>
+      <c r="AX21" s="282" t="n"/>
+      <c r="AY21" s="282" t="n"/>
+      <c r="AZ21" s="282" t="n"/>
+      <c r="BA21" s="282" t="n"/>
+      <c r="BB21" s="282" t="n"/>
+      <c r="BC21" s="282" t="n"/>
+      <c r="BD21" s="282" t="n"/>
+      <c r="BE21" s="288" t="n"/>
+      <c r="BF21" s="289" t="n"/>
+      <c r="BG21" s="156" t="n"/>
+      <c r="BH21" s="156" t="n"/>
+      <c r="BI21" s="156" t="n"/>
+      <c r="BJ21" s="156" t="n"/>
+      <c r="BK21" s="156" t="n"/>
+      <c r="BL21" s="156" t="n"/>
+      <c r="BM21" s="156" t="n"/>
+      <c r="BN21" s="156" t="n"/>
+      <c r="BO21" s="156" t="n"/>
+      <c r="BP21" s="153" t="n"/>
+      <c r="BQ21" s="153" t="n"/>
+      <c r="BR21" s="153" t="n"/>
+      <c r="BS21" s="153" t="n"/>
+      <c r="BT21" s="153" t="n"/>
+      <c r="BU21" s="153" t="n"/>
+      <c r="BV21" s="153" t="n"/>
+      <c r="BW21" s="153" t="n"/>
+      <c r="BX21" s="153" t="n"/>
+      <c r="BY21" s="153" t="n"/>
+      <c r="BZ21" s="153" t="n"/>
+      <c r="CA21" s="153" t="n"/>
     </row>
-    <row r="22" ht="20" customFormat="1" customHeight="1" s="53" thickBot="1">
-      <c r="A22" s="130" t="n"/>
-      <c r="B22" s="99" t="inlineStr">
+    <row r="22" ht="54" customFormat="1" customHeight="1" s="53" thickBot="1">
+      <c r="A22" s="197" t="n"/>
+      <c r="B22" s="247" t="inlineStr">
         <is>
           <t>Conclusion</t>
         </is>
       </c>
-      <c r="C22" s="100" t="n">
+      <c r="C22" s="248" t="n">
         <v>0</v>
       </c>
-      <c r="D22" s="83" t="n">
-        <v>46082</v>
-      </c>
-      <c r="E22" s="83" t="n">
-        <v>46174</v>
-      </c>
-      <c r="F22" s="84" t="n"/>
-      <c r="G22" s="85" t="n"/>
-      <c r="H22" s="86" t="n"/>
-      <c r="I22" s="86" t="n"/>
-      <c r="J22" s="86" t="n"/>
-      <c r="K22" s="86" t="n"/>
-      <c r="L22" s="86" t="n"/>
-      <c r="M22" s="86" t="n"/>
-      <c r="N22" s="86" t="n"/>
-      <c r="O22" s="86" t="n"/>
-      <c r="P22" s="86" t="n"/>
-      <c r="Q22" s="86" t="n"/>
-      <c r="R22" s="86" t="n"/>
-      <c r="S22" s="86" t="n"/>
-      <c r="T22" s="86" t="n"/>
-      <c r="U22" s="86" t="n"/>
-      <c r="V22" s="86" t="n"/>
-      <c r="W22" s="86" t="n"/>
-      <c r="X22" s="86" t="n"/>
-      <c r="Y22" s="86" t="n"/>
-      <c r="Z22" s="86" t="n"/>
-      <c r="AA22" s="86" t="n"/>
-      <c r="AB22" s="86" t="n"/>
-      <c r="AC22" s="86" t="n"/>
-      <c r="AD22" s="86" t="n"/>
-      <c r="AE22" s="86" t="n"/>
-      <c r="AF22" s="86" t="n"/>
-      <c r="AG22" s="86" t="n"/>
-      <c r="AH22" s="86" t="n"/>
-      <c r="AI22" s="86" t="n"/>
-      <c r="AJ22" s="86" t="n"/>
-      <c r="AK22" s="86" t="n"/>
-      <c r="AL22" s="86" t="n"/>
-      <c r="AM22" s="86" t="n"/>
-      <c r="AN22" s="86" t="n"/>
-      <c r="AO22" s="86" t="n"/>
-      <c r="AP22" s="86" t="n"/>
-      <c r="AQ22" s="86" t="n"/>
-      <c r="AR22" s="86" t="n"/>
-      <c r="AS22" s="86" t="n"/>
-      <c r="AT22" s="86" t="n"/>
-      <c r="AU22" s="86" t="n"/>
-      <c r="AV22" s="86" t="n"/>
-      <c r="AW22" s="86" t="n"/>
-      <c r="AX22" s="144" t="inlineStr">
+      <c r="D22" s="249" t="n">
+        <v>46117</v>
+      </c>
+      <c r="E22" s="249" t="n">
+        <v>46148</v>
+      </c>
+      <c r="F22" s="216" t="n"/>
+      <c r="G22" s="217" t="n"/>
+      <c r="H22" s="270" t="inlineStr">
         <is>
-          <t>Chp7:Conclusion</t>
+          <t>Chp 7 - Conclusion</t>
         </is>
       </c>
-      <c r="AY22" s="86" t="n"/>
-      <c r="AZ22" s="86" t="n"/>
-      <c r="BA22" s="86" t="n"/>
-      <c r="BB22" s="86" t="n"/>
-      <c r="BC22" s="86" t="n"/>
-      <c r="BD22" s="86" t="n"/>
-      <c r="BH22" s="55" t="n"/>
-      <c r="BI22" s="55" t="n"/>
-      <c r="BJ22" s="55" t="n"/>
-      <c r="BK22" s="55" t="n"/>
+      <c r="I22" s="282" t="n"/>
+      <c r="J22" s="282" t="n"/>
+      <c r="K22" s="282" t="n"/>
+      <c r="L22" s="282" t="n"/>
+      <c r="M22" s="282" t="n"/>
+      <c r="N22" s="282" t="n"/>
+      <c r="O22" s="282" t="n"/>
+      <c r="P22" s="282" t="n"/>
+      <c r="Q22" s="282" t="n"/>
+      <c r="R22" s="282" t="n"/>
+      <c r="S22" s="282" t="n"/>
+      <c r="T22" s="282" t="n"/>
+      <c r="U22" s="282" t="n"/>
+      <c r="V22" s="282" t="n"/>
+      <c r="W22" s="282" t="n"/>
+      <c r="X22" s="282" t="n"/>
+      <c r="Y22" s="282" t="n"/>
+      <c r="Z22" s="282" t="n"/>
+      <c r="AA22" s="282" t="n"/>
+      <c r="AB22" s="282" t="n"/>
+      <c r="AC22" s="282" t="n"/>
+      <c r="AD22" s="282" t="n"/>
+      <c r="AE22" s="282" t="n"/>
+      <c r="AF22" s="282" t="n"/>
+      <c r="AG22" s="282" t="n"/>
+      <c r="AH22" s="282" t="n"/>
+      <c r="AI22" s="282" t="n"/>
+      <c r="AJ22" s="282" t="n"/>
+      <c r="AK22" s="282" t="n"/>
+      <c r="AL22" s="282" t="n"/>
+      <c r="AM22" s="282" t="n"/>
+      <c r="AN22" s="282" t="n"/>
+      <c r="AO22" s="282" t="n"/>
+      <c r="AP22" s="282" t="n"/>
+      <c r="AQ22" s="282" t="n"/>
+      <c r="AR22" s="282" t="n"/>
+      <c r="AS22" s="282" t="n"/>
+      <c r="AT22" s="282" t="n"/>
+      <c r="AU22" s="282" t="n"/>
+      <c r="AV22" s="282" t="n"/>
+      <c r="AW22" s="282" t="n"/>
+      <c r="AX22" s="273" t="n"/>
+      <c r="AY22" s="275" t="n"/>
+      <c r="AZ22" s="282" t="n"/>
+      <c r="BA22" s="282" t="n"/>
+      <c r="BB22" s="282" t="n"/>
+      <c r="BC22" s="282" t="n"/>
+      <c r="BD22" s="282" t="n"/>
+      <c r="BE22" s="284" t="n"/>
+      <c r="BF22" s="284" t="n"/>
+      <c r="BG22" s="153" t="n"/>
+      <c r="BH22" s="156" t="n"/>
+      <c r="BI22" s="156" t="n"/>
+      <c r="BJ22" s="156" t="n"/>
+      <c r="BK22" s="156" t="n"/>
+      <c r="BL22" s="153" t="n"/>
+      <c r="BM22" s="153" t="n"/>
+      <c r="BN22" s="153" t="n"/>
+      <c r="BO22" s="153" t="n"/>
+      <c r="BP22" s="153" t="n"/>
+      <c r="BQ22" s="153" t="n"/>
+      <c r="BR22" s="153" t="n"/>
+      <c r="BS22" s="153" t="n"/>
+      <c r="BT22" s="153" t="n"/>
+      <c r="BU22" s="153" t="n"/>
+      <c r="BV22" s="153" t="n"/>
+      <c r="BW22" s="153" t="n"/>
+      <c r="BX22" s="153" t="n"/>
+      <c r="BY22" s="153" t="n"/>
+      <c r="BZ22" s="153" t="n"/>
+      <c r="CA22" s="153" t="n"/>
     </row>
-    <row r="23" ht="20" customFormat="1" customHeight="1" s="53" thickBot="1">
-      <c r="A23" s="129" t="n"/>
-      <c r="B23" s="22" t="n"/>
-      <c r="C23" s="81" t="n"/>
+    <row r="23" ht="48" customFormat="1" customHeight="1" s="53" thickBot="1">
+      <c r="A23" s="178" t="n"/>
+      <c r="B23" s="278" t="n"/>
+      <c r="C23" s="279" t="n"/>
       <c r="D23" s="78" t="n"/>
       <c r="E23" s="78" t="n"/>
-      <c r="F23" s="13" t="n"/>
-      <c r="G23" s="3">
+      <c r="F23" s="182" t="n"/>
+      <c r="G23" s="183">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v/>
       </c>
-      <c r="H23" s="64" t="n"/>
-      <c r="I23" s="64" t="n"/>
-      <c r="J23" s="64" t="n"/>
-      <c r="K23" s="64" t="n"/>
-      <c r="L23" s="64" t="n"/>
-      <c r="M23" s="64" t="n"/>
-      <c r="N23" s="64" t="n"/>
-      <c r="O23" s="64" t="n"/>
-      <c r="P23" s="64" t="n"/>
-      <c r="Q23" s="64" t="n"/>
-      <c r="R23" s="64" t="n"/>
-      <c r="S23" s="64" t="n"/>
-      <c r="T23" s="64" t="n"/>
-      <c r="U23" s="64" t="n"/>
-      <c r="V23" s="64" t="n"/>
-      <c r="W23" s="132" t="n"/>
-      <c r="X23" s="133" t="n"/>
-      <c r="Y23" s="133" t="n"/>
-      <c r="Z23" s="133" t="n"/>
-      <c r="AA23" s="133" t="n"/>
-      <c r="AB23" s="133" t="n"/>
-      <c r="AC23" s="133" t="n"/>
-      <c r="AD23" s="133" t="n"/>
-      <c r="AE23" s="133" t="n"/>
-      <c r="AF23" s="133" t="n"/>
-      <c r="AG23" s="134" t="n"/>
-      <c r="AH23" s="64" t="n"/>
-      <c r="AI23" s="64" t="n"/>
-      <c r="AJ23" s="64" t="n"/>
-      <c r="AK23" s="64" t="n"/>
-      <c r="AL23" s="64" t="n"/>
-      <c r="AM23" s="64" t="n"/>
-      <c r="AN23" s="64" t="n"/>
-      <c r="AO23" s="64" t="n"/>
-      <c r="AP23" s="64" t="n"/>
-      <c r="AQ23" s="64" t="n"/>
-      <c r="AR23" s="64" t="n"/>
-      <c r="AS23" s="64" t="n"/>
-      <c r="AT23" s="64" t="n"/>
-      <c r="AU23" s="64" t="n"/>
-      <c r="AV23" s="64" t="n"/>
-      <c r="AW23" s="64" t="n"/>
-      <c r="AX23" s="64" t="n"/>
-      <c r="AY23" s="64" t="n"/>
-      <c r="AZ23" s="64" t="n"/>
-      <c r="BA23" s="140" t="inlineStr">
-        <is>
-          <t>Chp8: Conclusions</t>
-        </is>
-      </c>
-      <c r="BB23" s="64" t="n"/>
-      <c r="BC23" s="64" t="n"/>
-      <c r="BD23" s="64" t="n"/>
-      <c r="BE23" s="34" t="n"/>
-      <c r="BF23" s="34" t="n"/>
-      <c r="BG23" s="34" t="n"/>
-      <c r="BH23" s="34" t="n"/>
-      <c r="BI23" s="34" t="n"/>
-      <c r="BJ23" s="34" t="n"/>
-      <c r="BK23" s="34" t="n"/>
-      <c r="BL23" s="34" t="n"/>
-      <c r="BM23" s="34" t="n"/>
-      <c r="BN23" s="34" t="n"/>
-      <c r="BO23" s="34" t="n"/>
+      <c r="H23" s="282" t="n"/>
+      <c r="I23" s="282" t="n"/>
+      <c r="J23" s="282" t="n"/>
+      <c r="K23" s="282" t="n"/>
+      <c r="L23" s="282" t="n"/>
+      <c r="M23" s="282" t="n"/>
+      <c r="N23" s="282" t="n"/>
+      <c r="O23" s="282" t="n"/>
+      <c r="P23" s="282" t="n"/>
+      <c r="Q23" s="282" t="n"/>
+      <c r="R23" s="282" t="n"/>
+      <c r="S23" s="282" t="n"/>
+      <c r="T23" s="282" t="n"/>
+      <c r="U23" s="282" t="n"/>
+      <c r="V23" s="282" t="n"/>
+      <c r="W23" s="290" t="n"/>
+      <c r="X23" s="284" t="n"/>
+      <c r="Y23" s="284" t="n"/>
+      <c r="Z23" s="284" t="n"/>
+      <c r="AA23" s="284" t="n"/>
+      <c r="AB23" s="284" t="n"/>
+      <c r="AC23" s="284" t="n"/>
+      <c r="AD23" s="284" t="n"/>
+      <c r="AE23" s="284" t="n"/>
+      <c r="AF23" s="284" t="n"/>
+      <c r="AG23" s="284" t="n"/>
+      <c r="AH23" s="282" t="n"/>
+      <c r="AI23" s="282" t="n"/>
+      <c r="AJ23" s="282" t="n"/>
+      <c r="AK23" s="282" t="n"/>
+      <c r="AL23" s="282" t="n"/>
+      <c r="AM23" s="282" t="n"/>
+      <c r="AN23" s="282" t="n"/>
+      <c r="AO23" s="282" t="n"/>
+      <c r="AP23" s="282" t="n"/>
+      <c r="AQ23" s="282" t="n"/>
+      <c r="AR23" s="282" t="n"/>
+      <c r="AS23" s="282" t="n"/>
+      <c r="AT23" s="282" t="n"/>
+      <c r="AU23" s="282" t="n"/>
+      <c r="AV23" s="282" t="n"/>
+      <c r="AW23" s="282" t="n"/>
+      <c r="AX23" s="282" t="n"/>
+      <c r="AY23" s="282" t="n"/>
+      <c r="AZ23" s="282" t="n"/>
+      <c r="BA23" s="273" t="n"/>
+      <c r="BB23" s="282" t="n"/>
+      <c r="BC23" s="282" t="n"/>
+      <c r="BD23" s="282" t="n"/>
+      <c r="BE23" s="293" t="n"/>
+      <c r="BF23" s="293" t="n"/>
+      <c r="BG23" s="156" t="n"/>
+      <c r="BH23" s="156" t="n"/>
+      <c r="BI23" s="156" t="n"/>
+      <c r="BJ23" s="156" t="n"/>
+      <c r="BK23" s="156" t="n"/>
+      <c r="BL23" s="156" t="n"/>
+      <c r="BM23" s="156" t="n"/>
+      <c r="BN23" s="156" t="n"/>
+      <c r="BO23" s="156" t="n"/>
+      <c r="BP23" s="153" t="n"/>
+      <c r="BQ23" s="153" t="n"/>
+      <c r="BR23" s="153" t="n"/>
+      <c r="BS23" s="153" t="n"/>
+      <c r="BT23" s="153" t="n"/>
+      <c r="BU23" s="153" t="n"/>
+      <c r="BV23" s="153" t="n"/>
+      <c r="BW23" s="153" t="n"/>
+      <c r="BX23" s="153" t="n"/>
+      <c r="BY23" s="153" t="n"/>
+      <c r="BZ23" s="153" t="n"/>
+      <c r="CA23" s="153" t="n"/>
     </row>
     <row r="24" ht="30" customHeight="1" s="127" thickBot="1">
       <c r="C24" s="82" t="n"/>
@@ -4520,37 +5512,36 @@
     <row r="499" s="127"/>
     <row r="500" s="127"/>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="14">
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="H4:K4"/>
     <mergeCell ref="E5:E6"/>
     <mergeCell ref="P2:Y2"/>
     <mergeCell ref="AJ4:AU4"/>
-    <mergeCell ref="B5:B6"/>
     <mergeCell ref="H2:N2"/>
     <mergeCell ref="D5:D6"/>
     <mergeCell ref="W23:AG23"/>
     <mergeCell ref="X4:AI4"/>
     <mergeCell ref="L4:W4"/>
-    <mergeCell ref="AV4:BG4"/>
+    <mergeCell ref="B5:B6"/>
     <mergeCell ref="H1:N1"/>
     <mergeCell ref="P1:Y1"/>
     <mergeCell ref="C5:C6"/>
   </mergeCells>
-  <conditionalFormatting sqref="H9:BD14">
-    <cfRule type="expression" priority="1" dxfId="9" stopIfTrue="1">
+  <conditionalFormatting sqref="H9:BF14">
+    <cfRule type="expression" priority="5" dxfId="9" stopIfTrue="1">
       <formula>AND($D9&lt;=H$6,$D9+ROUNDDOWN(($E9-$D9+1)*$C9,0)-1&gt;=H$6)</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="10" stopIfTrue="0">
-      <formula>AND($D9&lt;=H$6,$E9&gt;=H$6)</formula>
+    <cfRule type="expression" priority="6" dxfId="10" stopIfTrue="0">
+      <formula>AND(ISNUMBER(H$6),EOMONTH(H$6,-1)+1&lt;=$E9,EOMONTH(H$6,0)&gt;=$D9)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H16:BD22">
-    <cfRule type="expression" priority="3" dxfId="11" stopIfTrue="1">
+  <conditionalFormatting sqref="H16:BF22">
+    <cfRule type="expression" priority="7" dxfId="13" stopIfTrue="1">
       <formula>AND($D16&lt;=H$6,$D16+ROUNDDOWN(($E16-$D16+1)*$C16,0)-1&gt;=H$6)</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" dxfId="12" stopIfTrue="0">
-      <formula>AND($D16&lt;=H$6,$E16&gt;=H$6)</formula>
+    <cfRule type="expression" priority="8" dxfId="14" stopIfTrue="0">
+      <formula>AND(ISNUMBER(H$6),EOMONTH(H$6,-1)+1&lt;=$E16,EOMONTH(H$6,0)&gt;=$D16)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="11">
@@ -4570,7 +5561,7 @@
   </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.35" right="0.35" top="0.35" bottom="0.5" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" scale="100"/>
+  <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>
   <headerFooter differentFirst="1" scaleWithDoc="0">
     <oddHeader/>
     <oddFooter>&amp;L&amp;C&amp;R</oddFooter>

</xml_diff>